<commit_message>
Publish audited finance upgrades, corrected pairs research and Tableau source limits
</commit_message>
<xml_diff>
--- a/projects/finance-release/Fleet_Investment.xlsx
+++ b/projects/finance-release/Fleet_Investment.xlsx
@@ -2,12 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rb8d9c0fbe82f4d61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="Rca13d7ed57d748f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="3" r:id="Rd1b2733f1e0c49a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="4" r:id="R12d59b0f76ae4548"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actions" sheetId="5" r:id="Rdd76d6b289cc455b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit" sheetId="6" r:id="Rf3059832442b4716"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rc38e4d8ac1724b0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="R2dca583960034956"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="3" r:id="R99b6d23b3edb46d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="4" r:id="Re49c442043d64196"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="After Tax" sheetId="5" r:id="R891d4e7225bb4a48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Financing" sheetId="6" r:id="R25c2cd5c2231494c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actions" sheetId="7" r:id="Redec429e0f524777"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit" sheetId="8" r:id="R35298ddd51714354"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,7 +20,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="7">
+  <x:numFmts count="9">
     <x:numFmt numFmtId="200" formatCode="0.0%"/>
     <x:numFmt numFmtId="201" formatCode="$0.00"/>
     <x:numFmt numFmtId="202" formatCode="#,##0;(#,##0);&quot;-&quot;"/>
@@ -26,6 +28,8 @@
     <x:numFmt numFmtId="204" formatCode="0.000"/>
     <x:numFmt numFmtId="205" formatCode="0.0"/>
     <x:numFmt numFmtId="206" formatCode="0.00"/>
+    <x:numFmt numFmtId="207" formatCode="#,##0"/>
+    <x:numFmt numFmtId="208" formatCode="0"/>
   </x:numFmts>
   <x:fonts count="7">
     <x:font>
@@ -104,7 +108,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="40">
+  <x:cellXfs count="47">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -177,6 +181,19 @@
     <x:xf numFmtId="206" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="208" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -214,7 +231,7 @@
                 <a:ea typeface="Arial"/>
                 <a:cs typeface="Arial"/>
               </a:rPr>
-              <a:t>Five-year present value of net costs (USD)</a:t>
+              <a:t>Five-year after-tax present value (USD)</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -242,19 +259,8 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>PV net costs</c:v>
+            <c:v>After-tax PV costs</c:v>
           </c:tx>
-          <c:spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="17324D"/>
-            </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
-              <a:solidFill>
-                <a:srgbClr val="17324D"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </c:spPr>
           <c:cat>
             <c:strRef>
               <c:f>'Summary'!$C$7:$C$9</c:f>
@@ -392,7 +398,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R461bdbee74ca46a8"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R07cde9af656245f2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -712,7 +718,7 @@
         <x:v>Alternative</x:v>
       </x:c>
       <x:c r="D6" s="23" t="str">
-        <x:v>PV net costs</x:v>
+        <x:v>After-tax PV costs</x:v>
       </x:c>
       <x:c r="E6" s="23" t="str">
         <x:v>Upfront cash needed</x:v>
@@ -739,11 +745,11 @@
         <x:v>Keep</x:v>
       </x:c>
       <x:c r="D7" s="35" t="n">
-        <x:f>-SUM('Cash Flows'!D35:I35)</x:f>
-        <x:v>2257157.54530663</x:v>
+        <x:f>-SUM('After Tax'!D29:I29)</x:f>
+        <x:v>1674900.963813121</x:v>
       </x:c>
       <x:c r="E7" s="35" t="n">
-        <x:f>MAX(0,-'Cash Flows'!D12)</x:f>
+        <x:f>MAX(0,-'After Tax'!D11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F7" s="35" t="n">
@@ -770,16 +776,16 @@
         <x:v>Replace</x:v>
       </x:c>
       <x:c r="D8" s="35" t="n">
-        <x:f>-SUM('Cash Flows'!D36:I36)</x:f>
-        <x:v>1883459.6803651936</x:v>
+        <x:f>-SUM('After Tax'!D30:I30)</x:f>
+        <x:v>1447379.0688278498</x:v>
       </x:c>
       <x:c r="E8" s="35" t="n">
-        <x:f>MAX(0,-'Cash Flows'!D20)</x:f>
-        <x:v>660000</x:v>
+        <x:f>MAX(0,-'After Tax'!D18)</x:f>
+        <x:v>685500</x:v>
       </x:c>
       <x:c r="F8" s="35" t="n">
         <x:f>$D$7-D8</x:f>
-        <x:v>373697.86494143633</x:v>
+        <x:v>227521.89498527115</x:v>
       </x:c>
       <x:c r="G8" s="28" t="str">
         <x:f>IF(E8&lt;='Assumptions'!$G$22,"Yes","No")</x:f>
@@ -801,16 +807,16 @@
         <x:v>Lease</x:v>
       </x:c>
       <x:c r="D9" s="35" t="n">
-        <x:f>-SUM('Cash Flows'!D37:I37)</x:f>
-        <x:v>1898668.0136767486</x:v>
+        <x:f>-SUM('After Tax'!D31:I31)</x:f>
+        <x:v>1441460.9154614909</x:v>
       </x:c>
       <x:c r="E9" s="35" t="n">
-        <x:f>MAX(0,-'Cash Flows'!D28)</x:f>
+        <x:f>MAX(0,-'After Tax'!D25)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F9" s="35" t="n">
         <x:f>$D$7-D9</x:f>
-        <x:v>358489.53162988136</x:v>
+        <x:v>233440.0483516301</x:v>
       </x:c>
       <x:c r="G9" s="28" t="str">
         <x:f>IF(E9&lt;='Assumptions'!$G$22,"Yes","No")</x:f>
@@ -867,7 +873,7 @@
       </x:c>
       <x:c r="D12" s="1" t="str">
         <x:f>INDEX(C7:C9,MATCH(MIN(D7:D9),D7:D9,0))</x:f>
-        <x:v>Replace</x:v>
+        <x:v>Lease</x:v>
       </x:c>
       <x:c r="E12" s="1"/>
       <x:c r="F12" s="1"/>
@@ -885,11 +891,11 @@
       <x:c r="A13" s="1"/>
       <x:c r="B13" s="1"/>
       <x:c r="C13" s="1" t="str">
-        <x:v>Recommended alternative within budget</x:v>
+        <x:v>Recommended within budget</x:v>
       </x:c>
       <x:c r="D13" s="1" t="str">
         <x:f>IF(AND(G8="Yes",D8&lt;=D7,OR(G9="No",D8&lt;=D9)),"Replace",IF(AND(G9="Yes",D9&lt;D7),"Lease","Keep"))</x:f>
-        <x:v>Replace</x:v>
+        <x:v>Lease</x:v>
       </x:c>
       <x:c r="E13" s="1"/>
       <x:c r="F13" s="1"/>
@@ -1116,38 +1122,38 @@
     <x:row r="26" ht="22" customHeight="1">
       <x:c r="A26" s="1"/>
       <x:c r="B26" s="1"/>
-      <x:c r="C26" s="1" t="str">
-        <x:v>Pre-tax comparison. Depreciation and financing are excluded.</x:v>
-      </x:c>
-      <x:c r="D26" s="1"/>
-      <x:c r="E26" s="1"/>
-      <x:c r="F26" s="1"/>
-      <x:c r="G26" s="1"/>
-      <x:c r="H26" s="1"/>
-      <x:c r="I26" s="1"/>
-      <x:c r="J26" s="1"/>
-      <x:c r="K26" s="1"/>
-      <x:c r="L26" s="1"/>
-      <x:c r="M26" s="1"/>
-      <x:c r="N26" s="1"/>
-      <x:c r="O26" s="1"/>
+      <x:c r="C26" s="5" t="str">
+        <x:v>After-tax unlevered NPV. Separate financing schedule; assumed full tax usability.</x:v>
+      </x:c>
+      <x:c r="D26" s="5"/>
+      <x:c r="E26" s="5"/>
+      <x:c r="F26" s="5"/>
+      <x:c r="G26" s="5"/>
+      <x:c r="H26" s="5"/>
+      <x:c r="I26" s="5"/>
+      <x:c r="J26" s="5"/>
+      <x:c r="K26" s="5"/>
+      <x:c r="L26" s="5"/>
+      <x:c r="M26" s="5"/>
+      <x:c r="N26" s="5"/>
+      <x:c r="O26" s="5"/>
     </x:row>
     <x:row r="27" ht="22" customHeight="1">
       <x:c r="A27" s="1"/>
       <x:c r="B27" s="1"/>
-      <x:c r="C27" s="1"/>
-      <x:c r="D27" s="1"/>
-      <x:c r="E27" s="1"/>
-      <x:c r="F27" s="1"/>
-      <x:c r="G27" s="1"/>
-      <x:c r="H27" s="1"/>
-      <x:c r="I27" s="1"/>
-      <x:c r="J27" s="1"/>
-      <x:c r="K27" s="1"/>
-      <x:c r="L27" s="1"/>
-      <x:c r="M27" s="1"/>
-      <x:c r="N27" s="1"/>
-      <x:c r="O27" s="1"/>
+      <x:c r="C27" s="5"/>
+      <x:c r="D27" s="5"/>
+      <x:c r="E27" s="5"/>
+      <x:c r="F27" s="5"/>
+      <x:c r="G27" s="5"/>
+      <x:c r="H27" s="5"/>
+      <x:c r="I27" s="5"/>
+      <x:c r="J27" s="5"/>
+      <x:c r="K27" s="5"/>
+      <x:c r="L27" s="5"/>
+      <x:c r="M27" s="5"/>
+      <x:c r="N27" s="5"/>
+      <x:c r="O27" s="5"/>
     </x:row>
     <x:row r="28" ht="22" customHeight="1">
       <x:c r="A28" s="1"/>
@@ -1803,7 +1809,7 @@
     <x:mergeCell ref="C26:O27"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2592ee44419a4725"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc2daf1ac0fa42f1"/>
 </x:worksheet>
 </file>
 
@@ -1816,9 +1822,9 @@
     <x:col min="3" max="3" width="42" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="17" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="17" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="28" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="28" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="28" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="32" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="32" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="32" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="17" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="17" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="17" hidden="0" customWidth="1"/>
@@ -2459,7 +2465,7 @@
       <x:c r="F32" s="1"/>
       <x:c r="G32" s="26" t="n">
         <x:f>'Summary'!F8</x:f>
-        <x:v>373697.86494143633</x:v>
+        <x:v>227521.89498527115</x:v>
       </x:c>
       <x:c r="H32" s="32" t="n">
         <x:v>0.06</x:v>
@@ -2485,13 +2491,13 @@
       </x:c>
       <x:c r="H33" s="25" t="n">
         <x:f t="dataTable" ref="H33:J35" dt2D="1" r1="D8" r2="D23"/>
-        <x:v>330761.2459142802</x:v>
+        <x:v>202897.48503772728</x:v>
       </x:c>
       <x:c r="I33" s="25" t="n">
-        <x:v>272409.44368964713</x:v>
+        <x:v>151555.57904642937</x:v>
       </x:c>
       <x:c r="J33" s="25" t="n">
-        <x:v>219146.53921469976</x:v>
+        <x:v>104642.04795561638</x:v>
       </x:c>
       <x:c r="K33" s="1"/>
       <x:c r="L33" s="1"/>
@@ -2507,13 +2513,13 @@
         <x:v>22000</x:v>
       </x:c>
       <x:c r="H34" s="25" t="n">
-        <x:v>437739.62462435407</x:v>
+        <x:v>283131.2690702826</x:v>
       </x:c>
       <x:c r="I34" s="25" t="n">
-        <x:v>373697.86494143633</x:v>
+        <x:v>227521.89498527115</x:v>
       </x:c>
       <x:c r="J34" s="25" t="n">
-        <x:v>315208.94195668865</x:v>
+        <x:v>176688.85001210799</x:v>
       </x:c>
       <x:c r="K34" s="1"/>
       <x:c r="L34" s="1"/>
@@ -2529,13 +2535,13 @@
         <x:v>26000</x:v>
       </x:c>
       <x:c r="H35" s="25" t="n">
-        <x:v>544718.003334428</x:v>
+        <x:v>363365.05310283764</x:v>
       </x:c>
       <x:c r="I35" s="25" t="n">
-        <x:v>474986.28619322553</x:v>
+        <x:v>303488.2109241134</x:v>
       </x:c>
       <x:c r="J35" s="25" t="n">
-        <x:v>411271.34469867684</x:v>
+        <x:v>248735.65206859936</x:v>
       </x:c>
       <x:c r="K35" s="1"/>
       <x:c r="L35" s="1"/>
@@ -2572,7 +2578,7 @@
       <x:c r="A38" s="1"/>
       <x:c r="B38" s="1"/>
       <x:c r="C38" s="5" t="str">
-        <x:v>Synthetic USD assumptions. Pre-tax appraisal; identical service output.</x:v>
+        <x:v>Synthetic appraisal. Tax basis, transition and lease mileage are explicit.</x:v>
       </x:c>
       <x:c r="D38" s="5"/>
       <x:c r="E38" s="5"/>
@@ -2640,212 +2646,346 @@
       <x:c r="K42" s="1"/>
       <x:c r="L42" s="1"/>
     </x:row>
-    <x:row r="43" ht="22" customHeight="1">
+    <x:row r="43" ht="15" hidden="0" customHeight="1">
       <x:c r="A43" s="1"/>
       <x:c r="B43" s="1"/>
       <x:c r="C43" s="1"/>
       <x:c r="D43" s="1"/>
       <x:c r="E43" s="1"/>
-      <x:c r="F43" s="1"/>
-      <x:c r="G43" s="1"/>
-      <x:c r="H43" s="1"/>
-      <x:c r="I43" s="1"/>
+      <x:c r="F43" s="23" t="str">
+        <x:v>Expanded driver</x:v>
+      </x:c>
+      <x:c r="G43" s="23" t="str">
+        <x:v>Value</x:v>
+      </x:c>
+      <x:c r="H43" s="23" t="str">
+        <x:v>Synthetic assumption</x:v>
+      </x:c>
+      <x:c r="I43" s="44" t="str">
+        <x:v>Validated value</x:v>
+      </x:c>
       <x:c r="J43" s="1"/>
       <x:c r="K43" s="1"/>
       <x:c r="L43" s="1"/>
     </x:row>
-    <x:row r="44" ht="22" customHeight="1">
+    <x:row r="44" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A44" s="1"/>
       <x:c r="B44" s="1"/>
       <x:c r="C44" s="1"/>
       <x:c r="D44" s="1"/>
       <x:c r="E44" s="1"/>
-      <x:c r="F44" s="1"/>
-      <x:c r="G44" s="1"/>
-      <x:c r="H44" s="1"/>
-      <x:c r="I44" s="1"/>
+      <x:c r="F44" s="5" t="str">
+        <x:v>Tax rate</x:v>
+      </x:c>
+      <x:c r="G44" s="34" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="H44" s="5" t="str">
+        <x:v>Immediate use of deductions assumed</x:v>
+      </x:c>
+      <x:c r="I44" s="8" t="n">
+        <x:f>IF(AND(ISNUMBER(G44),G44&gt;=0,G44&lt;=1),G44,NA())</x:f>
+        <x:v>0.25</x:v>
+      </x:c>
       <x:c r="J44" s="1"/>
       <x:c r="K44" s="1"/>
       <x:c r="L44" s="1"/>
     </x:row>
-    <x:row r="45" ht="22" customHeight="1">
+    <x:row r="45" ht="15" hidden="0" customHeight="1">
       <x:c r="A45" s="1"/>
       <x:c r="B45" s="1"/>
       <x:c r="C45" s="1"/>
       <x:c r="D45" s="1"/>
       <x:c r="E45" s="1"/>
-      <x:c r="F45" s="1"/>
-      <x:c r="G45" s="1"/>
-      <x:c r="H45" s="1"/>
-      <x:c r="I45" s="1"/>
+      <x:c r="F45" s="5" t="str">
+        <x:v>Old tax basis / vehicle</x:v>
+      </x:c>
+      <x:c r="G45" s="33" t="n">
+        <x:v>15000</x:v>
+      </x:c>
+      <x:c r="H45" s="5" t="str">
+        <x:v>Remaining depreciable basis</x:v>
+      </x:c>
+      <x:c r="I45" s="18" t="n">
+        <x:f>IF(AND(ISNUMBER(G45),G45&gt;=0),G45,NA())</x:f>
+        <x:v>15000</x:v>
+      </x:c>
       <x:c r="J45" s="1"/>
       <x:c r="K45" s="1"/>
       <x:c r="L45" s="1"/>
     </x:row>
-    <x:row r="46" ht="22" customHeight="1">
+    <x:row r="46" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A46" s="1"/>
       <x:c r="B46" s="1"/>
       <x:c r="C46" s="1"/>
       <x:c r="D46" s="1"/>
       <x:c r="E46" s="1"/>
-      <x:c r="F46" s="1"/>
-      <x:c r="G46" s="1"/>
-      <x:c r="H46" s="1"/>
-      <x:c r="I46" s="1"/>
+      <x:c r="F46" s="5" t="str">
+        <x:v>New tax residual / vehicle</x:v>
+      </x:c>
+      <x:c r="G46" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H46" s="5" t="str">
+        <x:v>Five-year straight-line tax depreciation</x:v>
+      </x:c>
+      <x:c r="I46" s="18" t="n">
+        <x:f>IF(AND(ISNUMBER(G46),G46&gt;=0),G46,NA())</x:f>
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="J46" s="1"/>
       <x:c r="K46" s="1"/>
       <x:c r="L46" s="1"/>
     </x:row>
-    <x:row r="47" ht="22" customHeight="1">
+    <x:row r="47" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A47" s="1"/>
       <x:c r="B47" s="1"/>
       <x:c r="C47" s="1"/>
       <x:c r="D47" s="1"/>
       <x:c r="E47" s="1"/>
-      <x:c r="F47" s="1"/>
-      <x:c r="G47" s="1"/>
-      <x:c r="H47" s="1"/>
-      <x:c r="I47" s="1"/>
+      <x:c r="F47" s="5" t="str">
+        <x:v>Transition cash / vehicle</x:v>
+      </x:c>
+      <x:c r="G47" s="33" t="n">
+        <x:v>4000</x:v>
+      </x:c>
+      <x:c r="H47" s="5" t="str">
+        <x:v>Replacement / lease commissioning; deductible</x:v>
+      </x:c>
+      <x:c r="I47" s="18" t="n">
+        <x:f>IF(AND(ISNUMBER(G47),G47&gt;=0),G47,NA())</x:f>
+        <x:v>4000</x:v>
+      </x:c>
       <x:c r="J47" s="1"/>
       <x:c r="K47" s="1"/>
       <x:c r="L47" s="1"/>
     </x:row>
-    <x:row r="48" ht="22" customHeight="1">
+    <x:row r="48" ht="15" hidden="0" customHeight="1">
       <x:c r="A48" s="1"/>
       <x:c r="B48" s="1"/>
       <x:c r="C48" s="1"/>
       <x:c r="D48" s="1"/>
       <x:c r="E48" s="1"/>
-      <x:c r="F48" s="1"/>
-      <x:c r="G48" s="1"/>
-      <x:c r="H48" s="1"/>
-      <x:c r="I48" s="1"/>
+      <x:c r="F48" s="5" t="str">
+        <x:v>Lease included miles / vehicle</x:v>
+      </x:c>
+      <x:c r="G48" s="41" t="n">
+        <x:v>65000</x:v>
+      </x:c>
+      <x:c r="H48" s="5" t="str">
+        <x:v>Annual allowance</x:v>
+      </x:c>
+      <x:c r="I48" s="46" t="n">
+        <x:f>IF(AND(ISNUMBER(G48),G48&gt;=0),G48,NA())</x:f>
+        <x:v>65000</x:v>
+      </x:c>
       <x:c r="J48" s="1"/>
       <x:c r="K48" s="1"/>
       <x:c r="L48" s="1"/>
     </x:row>
-    <x:row r="49" ht="22" customHeight="1">
+    <x:row r="49" ht="15" hidden="0" customHeight="1">
       <x:c r="A49" s="1"/>
       <x:c r="B49" s="1"/>
       <x:c r="C49" s="1"/>
       <x:c r="D49" s="1"/>
       <x:c r="E49" s="1"/>
-      <x:c r="F49" s="1"/>
-      <x:c r="G49" s="1"/>
-      <x:c r="H49" s="1"/>
-      <x:c r="I49" s="1"/>
+      <x:c r="F49" s="5" t="str">
+        <x:v>Excess mileage charge</x:v>
+      </x:c>
+      <x:c r="G49" s="40" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="H49" s="5" t="str">
+        <x:v>USD per excess mile</x:v>
+      </x:c>
+      <x:c r="I49" s="12" t="n">
+        <x:f>IF(AND(ISNUMBER(G49),G49&gt;=0),G49,NA())</x:f>
+        <x:v>0.2</x:v>
+      </x:c>
       <x:c r="J49" s="1"/>
       <x:c r="K49" s="1"/>
       <x:c r="L49" s="1"/>
     </x:row>
-    <x:row r="50" ht="22" customHeight="1">
+    <x:row r="50" ht="15" hidden="0" customHeight="1">
       <x:c r="A50" s="1"/>
       <x:c r="B50" s="1"/>
       <x:c r="C50" s="1"/>
       <x:c r="D50" s="1"/>
       <x:c r="E50" s="1"/>
-      <x:c r="F50" s="1"/>
-      <x:c r="G50" s="1"/>
-      <x:c r="H50" s="1"/>
-      <x:c r="I50" s="1"/>
+      <x:c r="F50" s="5" t="str">
+        <x:v>Debt fraction of new purchase</x:v>
+      </x:c>
+      <x:c r="G50" s="34" t="n">
+        <x:v>0.7</x:v>
+      </x:c>
+      <x:c r="H50" s="5" t="str">
+        <x:v>Assumed loan; not approved</x:v>
+      </x:c>
+      <x:c r="I50" s="8" t="n">
+        <x:f>IF(AND(ISNUMBER(G50),G50&gt;=0,G50&lt;=1),G50,NA())</x:f>
+        <x:v>0.7</x:v>
+      </x:c>
       <x:c r="J50" s="1"/>
       <x:c r="K50" s="1"/>
       <x:c r="L50" s="1"/>
     </x:row>
-    <x:row r="51" ht="22" customHeight="1">
+    <x:row r="51" ht="15" hidden="0" customHeight="1">
       <x:c r="A51" s="1"/>
       <x:c r="B51" s="1"/>
       <x:c r="C51" s="1"/>
       <x:c r="D51" s="1"/>
       <x:c r="E51" s="1"/>
-      <x:c r="F51" s="1"/>
-      <x:c r="G51" s="1"/>
-      <x:c r="H51" s="1"/>
-      <x:c r="I51" s="1"/>
+      <x:c r="F51" s="5" t="str">
+        <x:v>Annual debt rate</x:v>
+      </x:c>
+      <x:c r="G51" s="34" t="n">
+        <x:v>0.075</x:v>
+      </x:c>
+      <x:c r="H51" s="5" t="str">
+        <x:v>Five-year level principal</x:v>
+      </x:c>
+      <x:c r="I51" s="8" t="n">
+        <x:f>IF(AND(ISNUMBER(G51),G51&gt;=0,G51&lt;=1),G51,NA())</x:f>
+        <x:v>0.075</x:v>
+      </x:c>
       <x:c r="J51" s="1"/>
       <x:c r="K51" s="1"/>
       <x:c r="L51" s="1"/>
     </x:row>
-    <x:row r="52" ht="22" customHeight="1">
+    <x:row r="52" ht="15" hidden="0" customHeight="1">
       <x:c r="A52" s="1"/>
       <x:c r="B52" s="1"/>
       <x:c r="C52" s="1"/>
       <x:c r="D52" s="1"/>
       <x:c r="E52" s="1"/>
-      <x:c r="F52" s="1"/>
-      <x:c r="G52" s="1"/>
-      <x:c r="H52" s="1"/>
-      <x:c r="I52" s="1"/>
+      <x:c r="F52" s="5" t="str">
+        <x:v>Debt origination fee</x:v>
+      </x:c>
+      <x:c r="G52" s="34" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="H52" s="5" t="str">
+        <x:v>Upfront financing cost</x:v>
+      </x:c>
+      <x:c r="I52" s="8" t="n">
+        <x:f>IF(AND(ISNUMBER(G52),G52&gt;=0,G52&lt;=1),G52,NA())</x:f>
+        <x:v>0.01</x:v>
+      </x:c>
       <x:c r="J52" s="1"/>
       <x:c r="K52" s="1"/>
       <x:c r="L52" s="1"/>
     </x:row>
-    <x:row r="53" ht="22" customHeight="1">
+    <x:row r="53" ht="15" hidden="0" customHeight="1">
       <x:c r="A53" s="1"/>
       <x:c r="B53" s="1"/>
       <x:c r="C53" s="1"/>
       <x:c r="D53" s="1"/>
       <x:c r="E53" s="1"/>
-      <x:c r="F53" s="1"/>
-      <x:c r="G53" s="1"/>
-      <x:c r="H53" s="1"/>
-      <x:c r="I53" s="1"/>
+      <x:c r="F53" s="5" t="str">
+        <x:v>Lease accounting discount</x:v>
+      </x:c>
+      <x:c r="G53" s="34" t="n">
+        <x:v>0.075</x:v>
+      </x:c>
+      <x:c r="H53" s="5" t="str">
+        <x:v>Annual end-of-year payments</x:v>
+      </x:c>
+      <x:c r="I53" s="8" t="n">
+        <x:f>IF(AND(ISNUMBER(G53),G53&gt;=0,G53&lt;=1),G53,NA())</x:f>
+        <x:v>0.075</x:v>
+      </x:c>
       <x:c r="J53" s="1"/>
       <x:c r="K53" s="1"/>
       <x:c r="L53" s="1"/>
     </x:row>
-    <x:row r="54" ht="22" customHeight="1">
+    <x:row r="54" ht="15" hidden="0" customHeight="1">
       <x:c r="A54" s="1"/>
       <x:c r="B54" s="1"/>
       <x:c r="C54" s="1"/>
       <x:c r="D54" s="1"/>
       <x:c r="E54" s="1"/>
-      <x:c r="F54" s="1"/>
-      <x:c r="G54" s="1"/>
-      <x:c r="H54" s="1"/>
-      <x:c r="I54" s="1"/>
+      <x:c r="F54" s="5" t="str">
+        <x:v>Lease non-deductible deposit</x:v>
+      </x:c>
+      <x:c r="G54" s="33" t="n">
+        <x:v>50000</x:v>
+      </x:c>
+      <x:c r="H54" s="5" t="str">
+        <x:v>Returned at year five</x:v>
+      </x:c>
+      <x:c r="I54" s="18" t="n">
+        <x:f>IF(AND(ISNUMBER(G54),G54&gt;=0),G54,NA())</x:f>
+        <x:v>50000</x:v>
+      </x:c>
       <x:c r="J54" s="1"/>
       <x:c r="K54" s="1"/>
       <x:c r="L54" s="1"/>
     </x:row>
-    <x:row r="55" ht="22" customHeight="1">
+    <x:row r="55" ht="15" hidden="0" customHeight="1">
       <x:c r="A55" s="1"/>
       <x:c r="B55" s="1"/>
       <x:c r="C55" s="1"/>
       <x:c r="D55" s="1"/>
       <x:c r="E55" s="1"/>
-      <x:c r="F55" s="1"/>
-      <x:c r="G55" s="1"/>
-      <x:c r="H55" s="1"/>
-      <x:c r="I55" s="1"/>
+      <x:c r="F55" s="5" t="str">
+        <x:v>Tax depreciation years</x:v>
+      </x:c>
+      <x:c r="G55" s="42" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H55" s="5" t="str">
+        <x:v>No bonus depreciation</x:v>
+      </x:c>
+      <x:c r="I55" s="45" t="n">
+        <x:f>IF(AND(ISNUMBER(G55),G55&gt;=0,MOD(G55,1)=0,G55&gt;0),G55,NA())</x:f>
+        <x:v>5</x:v>
+      </x:c>
       <x:c r="J55" s="1"/>
       <x:c r="K55" s="1"/>
       <x:c r="L55" s="1"/>
     </x:row>
-    <x:row r="56" ht="22" customHeight="1">
+    <x:row r="56" ht="15" hidden="0" customHeight="1">
       <x:c r="A56" s="1"/>
       <x:c r="B56" s="1"/>
       <x:c r="C56" s="1"/>
       <x:c r="D56" s="1"/>
       <x:c r="E56" s="1"/>
-      <x:c r="F56" s="1"/>
-      <x:c r="G56" s="1"/>
-      <x:c r="H56" s="1"/>
-      <x:c r="I56" s="1"/>
+      <x:c r="F56" s="5" t="str">
+        <x:v>Transition deduction fraction</x:v>
+      </x:c>
+      <x:c r="G56" s="34" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H56" s="5" t="str">
+        <x:v>Sensitivity input</x:v>
+      </x:c>
+      <x:c r="I56" s="8" t="n">
+        <x:f>IF(AND(ISNUMBER(G56),G56&gt;=0,G56&lt;=1),G56,NA())</x:f>
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="J56" s="1"/>
       <x:c r="K56" s="1"/>
       <x:c r="L56" s="1"/>
     </x:row>
-    <x:row r="57" ht="22" customHeight="1">
+    <x:row r="57" ht="15" hidden="0" customHeight="1">
       <x:c r="A57" s="1"/>
       <x:c r="B57" s="1"/>
       <x:c r="C57" s="1"/>
       <x:c r="D57" s="1"/>
       <x:c r="E57" s="1"/>
-      <x:c r="F57" s="1"/>
-      <x:c r="G57" s="1"/>
-      <x:c r="H57" s="1"/>
-      <x:c r="I57" s="1"/>
+      <x:c r="F57" s="5" t="str">
+        <x:v>Tax usable fraction</x:v>
+      </x:c>
+      <x:c r="G57" s="34" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H57" s="5" t="str">
+        <x:v>Set zero when deductions unusable</x:v>
+      </x:c>
+      <x:c r="I57" s="8" t="n">
+        <x:f>IF(AND(ISNUMBER(G57),G57&gt;=0,G57&lt;=1),G57,NA())</x:f>
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="J57" s="1"/>
       <x:c r="K57" s="1"/>
       <x:c r="L57" s="1"/>
@@ -3013,7 +3153,7 @@
       <x:c r="A2" s="1"/>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="2" t="str">
-        <x:v>Five-year fleet cash flows</x:v>
+        <x:v>Pre-tax operating cash flows</x:v>
       </x:c>
       <x:c r="D2" s="1"/>
       <x:c r="E2" s="1"/>
@@ -4626,7 +4766,7 @@
       <x:c r="A13" s="1"/>
       <x:c r="B13" s="1"/>
       <x:c r="C13" s="5" t="str">
-        <x:v>Simulated review only. Annualized observations are not realized employer savings.</x:v>
+        <x:v>Legacy simulated observations are preserved. The $660k target uses the original pre-tax scope.</x:v>
       </x:c>
       <x:c r="D13" s="5"/>
       <x:c r="E13" s="5"/>
@@ -5380,13 +5520,13 @@
   <x:cols>
     <x:col min="1" max="1" width="3" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="3" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="27" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="27" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="27" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="27" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="27" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="27" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="27" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="42" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="17" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="17" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="17" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="17" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="17" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="17" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="17" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="17" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="17" hidden="0" customWidth="1"/>
@@ -5410,7 +5550,7 @@
       <x:c r="A2" s="1"/>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="2" t="str">
-        <x:v>Decision ownership and approval</x:v>
+        <x:v>After-tax unlevered alternatives</x:v>
       </x:c>
       <x:c r="D2" s="1"/>
       <x:c r="E2" s="1"/>
@@ -5440,9 +5580,12 @@
       <x:c r="A4" s="1"/>
       <x:c r="B4" s="1"/>
       <x:c r="C4" s="1" t="str">
-        <x:v>Roles and deadlines are proposed within a synthetic case.</x:v>
-      </x:c>
-      <x:c r="D4" s="1"/>
+        <x:v>Case selected</x:v>
+      </x:c>
+      <x:c r="D4" s="7" t="str">
+        <x:f>'Assumptions'!D4</x:f>
+        <x:v>Base</x:v>
+      </x:c>
       <x:c r="E4" s="1"/>
       <x:c r="F4" s="1"/>
       <x:c r="G4" s="1"/>
@@ -5466,134 +5609,152 @@
       <x:c r="K5" s="1"/>
       <x:c r="L5" s="1"/>
     </x:row>
-    <x:row r="6" ht="15" hidden="0" customHeight="1">
+    <x:row r="6" ht="22" customHeight="1">
       <x:c r="A6" s="1"/>
       <x:c r="B6" s="1"/>
-      <x:c r="C6" s="23" t="str">
-        <x:v>Action</x:v>
-      </x:c>
-      <x:c r="D6" s="23" t="str">
-        <x:v>Proposed owner</x:v>
-      </x:c>
-      <x:c r="E6" s="23" t="str">
-        <x:v>Due from approval</x:v>
-      </x:c>
-      <x:c r="F6" s="23" t="str">
-        <x:v>Trigger / evidence</x:v>
-      </x:c>
-      <x:c r="G6" s="23" t="str">
-        <x:v>Approval needed</x:v>
-      </x:c>
-      <x:c r="H6" s="23" t="str">
-        <x:v>Status</x:v>
-      </x:c>
-      <x:c r="I6" s="23" t="str">
-        <x:v>Evidence link</x:v>
+      <x:c r="C6" s="1"/>
+      <x:c r="D6" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E6" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F6" s="4" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G6" s="4" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H6" s="4" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I6" s="4" t="n">
+        <x:v>5</x:v>
       </x:c>
       <x:c r="J6" s="1"/>
       <x:c r="K6" s="1"/>
       <x:c r="L6" s="1"/>
     </x:row>
-    <x:row r="7" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="7" ht="22" customHeight="1">
       <x:c r="A7" s="1"/>
       <x:c r="B7" s="1"/>
-      <x:c r="C7" s="5" t="str">
-        <x:v>Obtain purchase and lease quotes</x:v>
-      </x:c>
-      <x:c r="D7" s="5" t="str">
-        <x:v>Fleet + Procurement</x:v>
-      </x:c>
-      <x:c r="E7" s="5" t="str">
-        <x:v>Day 10</x:v>
-      </x:c>
-      <x:c r="F7" s="5" t="str">
-        <x:v>Comparable service and coverage</x:v>
-      </x:c>
-      <x:c r="G7" s="5" t="str">
-        <x:v>Procurement lead</x:v>
-      </x:c>
-      <x:c r="H7" s="5" t="str">
-        <x:v>Proposed</x:v>
-      </x:c>
-      <x:c r="I7" s="5" t="str"/>
+      <x:c r="C7" s="1" t="str">
+        <x:v>Keep operating cash costs</x:v>
+      </x:c>
+      <x:c r="D7" s="25"/>
+      <x:c r="E7" s="26" t="n">
+        <x:f>'Cash Flows'!E10</x:f>
+        <x:v>541600</x:v>
+      </x:c>
+      <x:c r="F7" s="26" t="n">
+        <x:f>'Cash Flows'!F10</x:f>
+        <x:v>557848</x:v>
+      </x:c>
+      <x:c r="G7" s="26" t="n">
+        <x:f>'Cash Flows'!G10</x:f>
+        <x:v>574583.44</x:v>
+      </x:c>
+      <x:c r="H7" s="26" t="n">
+        <x:f>'Cash Flows'!H10</x:f>
+        <x:v>591820.9432</x:v>
+      </x:c>
+      <x:c r="I7" s="26" t="n">
+        <x:f>'Cash Flows'!I10</x:f>
+        <x:v>609575.571496</x:v>
+      </x:c>
       <x:c r="J7" s="1"/>
       <x:c r="K7" s="1"/>
       <x:c r="L7" s="1"/>
     </x:row>
-    <x:row r="8" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="8" ht="22" customHeight="1">
       <x:c r="A8" s="1"/>
       <x:c r="B8" s="1"/>
-      <x:c r="C8" s="5" t="str">
-        <x:v>Approve capital and liquidity</x:v>
-      </x:c>
-      <x:c r="D8" s="5" t="str">
-        <x:v>Finance + Treasury</x:v>
-      </x:c>
-      <x:c r="E8" s="5" t="str">
-        <x:v>Day 15</x:v>
-      </x:c>
-      <x:c r="F8" s="5" t="str">
-        <x:v>Net upfront cash within $700k</x:v>
-      </x:c>
-      <x:c r="G8" s="5" t="str">
-        <x:v>Investment committee</x:v>
-      </x:c>
-      <x:c r="H8" s="5" t="str">
-        <x:v>Proposed</x:v>
-      </x:c>
-      <x:c r="I8" s="5" t="str"/>
+      <x:c r="C8" s="1" t="str">
+        <x:v>Keep tax depreciation</x:v>
+      </x:c>
+      <x:c r="D8" s="25"/>
+      <x:c r="E8" s="26" t="n">
+        <x:f>'Assumptions'!$G$9*'Assumptions'!$I$45/'Assumptions'!$I$55</x:f>
+        <x:v>18000</x:v>
+      </x:c>
+      <x:c r="F8" s="26" t="n">
+        <x:f>'Assumptions'!$G$9*'Assumptions'!$I$45/'Assumptions'!$I$55</x:f>
+        <x:v>18000</x:v>
+      </x:c>
+      <x:c r="G8" s="26" t="n">
+        <x:f>'Assumptions'!$G$9*'Assumptions'!$I$45/'Assumptions'!$I$55</x:f>
+        <x:v>18000</x:v>
+      </x:c>
+      <x:c r="H8" s="26" t="n">
+        <x:f>'Assumptions'!$G$9*'Assumptions'!$I$45/'Assumptions'!$I$55</x:f>
+        <x:v>18000</x:v>
+      </x:c>
+      <x:c r="I8" s="26" t="n">
+        <x:f>'Assumptions'!$G$9*'Assumptions'!$I$45/'Assumptions'!$I$55</x:f>
+        <x:v>18000</x:v>
+      </x:c>
       <x:c r="J8" s="1"/>
       <x:c r="K8" s="1"/>
       <x:c r="L8" s="1"/>
     </x:row>
-    <x:row r="9" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="9" ht="22" customHeight="1">
       <x:c r="A9" s="1"/>
       <x:c r="B9" s="1"/>
-      <x:c r="C9" s="5" t="str">
-        <x:v>Verify tax and residual assumptions</x:v>
-      </x:c>
-      <x:c r="D9" s="5" t="str">
-        <x:v>Finance</x:v>
-      </x:c>
-      <x:c r="E9" s="5" t="str">
-        <x:v>Before commitment</x:v>
-      </x:c>
-      <x:c r="F9" s="5" t="str">
-        <x:v>Tax-adjusted economics reviewed</x:v>
-      </x:c>
-      <x:c r="G9" s="5" t="str">
-        <x:v>Finance lead</x:v>
-      </x:c>
-      <x:c r="H9" s="5" t="str">
-        <x:v>Proposed</x:v>
-      </x:c>
-      <x:c r="I9" s="5" t="str"/>
+      <x:c r="C9" s="1" t="str">
+        <x:v>Keep tax benefit</x:v>
+      </x:c>
+      <x:c r="D9" s="25"/>
+      <x:c r="E9" s="26" t="n">
+        <x:f>SUM(E7:E8)*'Assumptions'!$I$44*'Assumptions'!$I$57</x:f>
+        <x:v>139900</x:v>
+      </x:c>
+      <x:c r="F9" s="26" t="n">
+        <x:f>SUM(F7:F8)*'Assumptions'!$I$44*'Assumptions'!$I$57</x:f>
+        <x:v>143962</x:v>
+      </x:c>
+      <x:c r="G9" s="26" t="n">
+        <x:f>SUM(G7:G8)*'Assumptions'!$I$44*'Assumptions'!$I$57</x:f>
+        <x:v>148145.86</x:v>
+      </x:c>
+      <x:c r="H9" s="26" t="n">
+        <x:f>SUM(H7:H8)*'Assumptions'!$I$44*'Assumptions'!$I$57</x:f>
+        <x:v>152455.2358</x:v>
+      </x:c>
+      <x:c r="I9" s="26" t="n">
+        <x:f>SUM(I7:I8)*'Assumptions'!$I$44*'Assumptions'!$I$57</x:f>
+        <x:v>156893.892874</x:v>
+      </x:c>
       <x:c r="J9" s="1"/>
       <x:c r="K9" s="1"/>
       <x:c r="L9" s="1"/>
     </x:row>
-    <x:row r="10" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="10" ht="22" customHeight="1">
       <x:c r="A10" s="1"/>
       <x:c r="B10" s="1"/>
-      <x:c r="C10" s="5" t="str">
-        <x:v>Review benefits after commissioning</x:v>
-      </x:c>
-      <x:c r="D10" s="5" t="str">
-        <x:v>Fleet + Finance</x:v>
-      </x:c>
-      <x:c r="E10" s="5" t="str">
-        <x:v>Days 30 / 90 / 180</x:v>
-      </x:c>
-      <x:c r="F10" s="5" t="str">
-        <x:v>Maintenance, mpg, downtime vs plan</x:v>
-      </x:c>
-      <x:c r="G10" s="5" t="str">
-        <x:v>Operations lead</x:v>
-      </x:c>
-      <x:c r="H10" s="5" t="str">
-        <x:v>Proposed</x:v>
-      </x:c>
-      <x:c r="I10" s="5" t="str"/>
+      <x:c r="C10" s="1" t="str">
+        <x:v>Keep after-tax terminal value</x:v>
+      </x:c>
+      <x:c r="D10" s="25"/>
+      <x:c r="E10" s="18" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F10" s="18" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G10" s="18" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H10" s="18" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I10" s="26" t="n">
+        <x:f>'Cash Flows'!I11*(1-'Assumptions'!I44)</x:f>
+        <x:v>31500</x:v>
+      </x:c>
       <x:c r="J10" s="1"/>
       <x:c r="K10" s="1"/>
       <x:c r="L10" s="1"/>
@@ -5601,13 +5762,33 @@
     <x:row r="11" ht="22" customHeight="1">
       <x:c r="A11" s="1"/>
       <x:c r="B11" s="1"/>
-      <x:c r="C11" s="1"/>
-      <x:c r="D11" s="1"/>
-      <x:c r="E11" s="1"/>
-      <x:c r="F11" s="1"/>
-      <x:c r="G11" s="1"/>
-      <x:c r="H11" s="1"/>
-      <x:c r="I11" s="1"/>
+      <x:c r="C11" s="1" t="str">
+        <x:v>Keep unlevered cash flow</x:v>
+      </x:c>
+      <x:c r="D11" s="18" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E11" s="18" t="n">
+        <x:f>-E7+SUM(E9:E10)</x:f>
+        <x:v>-401700</x:v>
+      </x:c>
+      <x:c r="F11" s="18" t="n">
+        <x:f>-F7+SUM(F9:F10)</x:f>
+        <x:v>-413886</x:v>
+      </x:c>
+      <x:c r="G11" s="18" t="n">
+        <x:f>-G7+SUM(G9:G10)</x:f>
+        <x:v>-426437.57999999996</x:v>
+      </x:c>
+      <x:c r="H11" s="18" t="n">
+        <x:f>-H7+SUM(H9:H10)</x:f>
+        <x:v>-439365.70739999996</x:v>
+      </x:c>
+      <x:c r="I11" s="18" t="n">
+        <x:f>-I7+SUM(I9:I10)</x:f>
+        <x:v>-421181.67862200004</x:v>
+      </x:c>
       <x:c r="J11" s="1"/>
       <x:c r="K11" s="1"/>
       <x:c r="L11" s="1"/>
@@ -5616,12 +5797,12 @@
       <x:c r="A12" s="1"/>
       <x:c r="B12" s="1"/>
       <x:c r="C12" s="1"/>
-      <x:c r="D12" s="1"/>
-      <x:c r="E12" s="1"/>
-      <x:c r="F12" s="1"/>
-      <x:c r="G12" s="1"/>
-      <x:c r="H12" s="1"/>
-      <x:c r="I12" s="1"/>
+      <x:c r="D12" s="25"/>
+      <x:c r="E12" s="25"/>
+      <x:c r="F12" s="25"/>
+      <x:c r="G12" s="25"/>
+      <x:c r="H12" s="25"/>
+      <x:c r="I12" s="25"/>
       <x:c r="J12" s="1"/>
       <x:c r="K12" s="1"/>
       <x:c r="L12" s="1"/>
@@ -5630,12 +5811,12 @@
       <x:c r="A13" s="1"/>
       <x:c r="B13" s="1"/>
       <x:c r="C13" s="1"/>
-      <x:c r="D13" s="1"/>
-      <x:c r="E13" s="1"/>
-      <x:c r="F13" s="1"/>
-      <x:c r="G13" s="1"/>
-      <x:c r="H13" s="1"/>
-      <x:c r="I13" s="1"/>
+      <x:c r="D13" s="25"/>
+      <x:c r="E13" s="25"/>
+      <x:c r="F13" s="25"/>
+      <x:c r="G13" s="25"/>
+      <x:c r="H13" s="25"/>
+      <x:c r="I13" s="25"/>
       <x:c r="J13" s="1"/>
       <x:c r="K13" s="1"/>
       <x:c r="L13" s="1"/>
@@ -5643,13 +5824,30 @@
     <x:row r="14" ht="22" customHeight="1">
       <x:c r="A14" s="1"/>
       <x:c r="B14" s="1"/>
-      <x:c r="C14" s="1"/>
-      <x:c r="D14" s="1"/>
-      <x:c r="E14" s="1"/>
-      <x:c r="F14" s="1"/>
-      <x:c r="G14" s="1"/>
-      <x:c r="H14" s="1"/>
-      <x:c r="I14" s="1"/>
+      <x:c r="C14" s="1" t="str">
+        <x:v>Replace operating cash costs</x:v>
+      </x:c>
+      <x:c r="D14" s="25"/>
+      <x:c r="E14" s="26" t="n">
+        <x:f>'Cash Flows'!E18</x:f>
+        <x:v>330533.3333333333</x:v>
+      </x:c>
+      <x:c r="F14" s="26" t="n">
+        <x:f>'Cash Flows'!F18</x:f>
+        <x:v>340449.3333333333</x:v>
+      </x:c>
+      <x:c r="G14" s="26" t="n">
+        <x:f>'Cash Flows'!G18</x:f>
+        <x:v>350662.8133333333</x:v>
+      </x:c>
+      <x:c r="H14" s="26" t="n">
+        <x:f>'Cash Flows'!H18</x:f>
+        <x:v>361182.69773333333</x:v>
+      </x:c>
+      <x:c r="I14" s="26" t="n">
+        <x:f>'Cash Flows'!I18</x:f>
+        <x:v>372018.17866533337</x:v>
+      </x:c>
       <x:c r="J14" s="1"/>
       <x:c r="K14" s="1"/>
       <x:c r="L14" s="1"/>
@@ -5657,13 +5855,30 @@
     <x:row r="15" ht="22" customHeight="1">
       <x:c r="A15" s="1"/>
       <x:c r="B15" s="1"/>
-      <x:c r="C15" s="1"/>
-      <x:c r="D15" s="1"/>
-      <x:c r="E15" s="1"/>
-      <x:c r="F15" s="1"/>
-      <x:c r="G15" s="1"/>
-      <x:c r="H15" s="1"/>
-      <x:c r="I15" s="1"/>
+      <x:c r="C15" s="1" t="str">
+        <x:v>Replace tax depreciation</x:v>
+      </x:c>
+      <x:c r="D15" s="25"/>
+      <x:c r="E15" s="26" t="n">
+        <x:f>'Assumptions'!$G$9*('Assumptions'!$G$10-'Assumptions'!$I$46)/'Assumptions'!$I$55</x:f>
+        <x:v>156000</x:v>
+      </x:c>
+      <x:c r="F15" s="26" t="n">
+        <x:f>'Assumptions'!$G$9*('Assumptions'!$G$10-'Assumptions'!$I$46)/'Assumptions'!$I$55</x:f>
+        <x:v>156000</x:v>
+      </x:c>
+      <x:c r="G15" s="26" t="n">
+        <x:f>'Assumptions'!$G$9*('Assumptions'!$G$10-'Assumptions'!$I$46)/'Assumptions'!$I$55</x:f>
+        <x:v>156000</x:v>
+      </x:c>
+      <x:c r="H15" s="26" t="n">
+        <x:f>'Assumptions'!$G$9*('Assumptions'!$G$10-'Assumptions'!$I$46)/'Assumptions'!$I$55</x:f>
+        <x:v>156000</x:v>
+      </x:c>
+      <x:c r="I15" s="26" t="n">
+        <x:f>'Assumptions'!$G$9*('Assumptions'!$G$10-'Assumptions'!$I$46)/'Assumptions'!$I$55</x:f>
+        <x:v>156000</x:v>
+      </x:c>
       <x:c r="J15" s="1"/>
       <x:c r="K15" s="1"/>
       <x:c r="L15" s="1"/>
@@ -5671,13 +5886,30 @@
     <x:row r="16" ht="22" customHeight="1">
       <x:c r="A16" s="1"/>
       <x:c r="B16" s="1"/>
-      <x:c r="C16" s="1"/>
-      <x:c r="D16" s="1"/>
-      <x:c r="E16" s="1"/>
-      <x:c r="F16" s="1"/>
-      <x:c r="G16" s="1"/>
-      <x:c r="H16" s="1"/>
-      <x:c r="I16" s="1"/>
+      <x:c r="C16" s="1" t="str">
+        <x:v>Replace tax benefit</x:v>
+      </x:c>
+      <x:c r="D16" s="25"/>
+      <x:c r="E16" s="26" t="n">
+        <x:f>SUM(E14:E15)*'Assumptions'!$I$44*'Assumptions'!$I$57</x:f>
+        <x:v>121633.33333333333</x:v>
+      </x:c>
+      <x:c r="F16" s="26" t="n">
+        <x:f>SUM(F14:F15)*'Assumptions'!$I$44*'Assumptions'!$I$57</x:f>
+        <x:v>124112.33333333333</x:v>
+      </x:c>
+      <x:c r="G16" s="26" t="n">
+        <x:f>SUM(G14:G15)*'Assumptions'!$I$44*'Assumptions'!$I$57</x:f>
+        <x:v>126665.70333333332</x:v>
+      </x:c>
+      <x:c r="H16" s="26" t="n">
+        <x:f>SUM(H14:H15)*'Assumptions'!$I$44*'Assumptions'!$I$57</x:f>
+        <x:v>129295.67443333333</x:v>
+      </x:c>
+      <x:c r="I16" s="26" t="n">
+        <x:f>SUM(I14:I15)*'Assumptions'!$I$44*'Assumptions'!$I$57</x:f>
+        <x:v>132004.54466633336</x:v>
+      </x:c>
       <x:c r="J16" s="1"/>
       <x:c r="K16" s="1"/>
       <x:c r="L16" s="1"/>
@@ -5685,13 +5917,30 @@
     <x:row r="17" ht="22" customHeight="1">
       <x:c r="A17" s="1"/>
       <x:c r="B17" s="1"/>
-      <x:c r="C17" s="1"/>
-      <x:c r="D17" s="1"/>
-      <x:c r="E17" s="1"/>
-      <x:c r="F17" s="1"/>
-      <x:c r="G17" s="1"/>
-      <x:c r="H17" s="1"/>
-      <x:c r="I17" s="1"/>
+      <x:c r="C17" s="1" t="str">
+        <x:v>Replace after-tax terminal value</x:v>
+      </x:c>
+      <x:c r="D17" s="25"/>
+      <x:c r="E17" s="18" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F17" s="18" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G17" s="18" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H17" s="18" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I17" s="26" t="n">
+        <x:f>'Cash Flows'!I19-('Cash Flows'!I19-'Assumptions'!G9*'Assumptions'!I46)*'Assumptions'!I44</x:f>
+        <x:v>189000</x:v>
+      </x:c>
       <x:c r="J17" s="1"/>
       <x:c r="K17" s="1"/>
       <x:c r="L17" s="1"/>
@@ -5699,13 +5948,33 @@
     <x:row r="18" ht="22" customHeight="1">
       <x:c r="A18" s="1"/>
       <x:c r="B18" s="1"/>
-      <x:c r="C18" s="1"/>
-      <x:c r="D18" s="1"/>
-      <x:c r="E18" s="1"/>
-      <x:c r="F18" s="1"/>
-      <x:c r="G18" s="1"/>
-      <x:c r="H18" s="1"/>
-      <x:c r="I18" s="1"/>
+      <x:c r="C18" s="1" t="str">
+        <x:v>Replace unlevered cash flow</x:v>
+      </x:c>
+      <x:c r="D18" s="26" t="n">
+        <x:f>'Cash Flows'!D20-('Assumptions'!G9*('Assumptions'!G11-'Assumptions'!I45))*'Assumptions'!I44-'Assumptions'!G9*'Assumptions'!I47*(1-'Assumptions'!I44*'Assumptions'!I56*'Assumptions'!I57)</x:f>
+        <x:v>-685500</x:v>
+      </x:c>
+      <x:c r="E18" s="18" t="n">
+        <x:f>-E14+SUM(E16:E17)</x:f>
+        <x:v>-208900</x:v>
+      </x:c>
+      <x:c r="F18" s="18" t="n">
+        <x:f>-F14+SUM(F16:F17)</x:f>
+        <x:v>-216337</x:v>
+      </x:c>
+      <x:c r="G18" s="18" t="n">
+        <x:f>-G14+SUM(G16:G17)</x:f>
+        <x:v>-223997.11</x:v>
+      </x:c>
+      <x:c r="H18" s="18" t="n">
+        <x:f>-H14+SUM(H16:H17)</x:f>
+        <x:v>-231887.0233</x:v>
+      </x:c>
+      <x:c r="I18" s="18" t="n">
+        <x:f>-I14+SUM(I16:I17)</x:f>
+        <x:v>-51013.63399900001</x:v>
+      </x:c>
       <x:c r="J18" s="1"/>
       <x:c r="K18" s="1"/>
       <x:c r="L18" s="1"/>
@@ -5714,12 +5983,12 @@
       <x:c r="A19" s="1"/>
       <x:c r="B19" s="1"/>
       <x:c r="C19" s="1"/>
-      <x:c r="D19" s="1"/>
-      <x:c r="E19" s="1"/>
-      <x:c r="F19" s="1"/>
-      <x:c r="G19" s="1"/>
-      <x:c r="H19" s="1"/>
-      <x:c r="I19" s="1"/>
+      <x:c r="D19" s="25"/>
+      <x:c r="E19" s="25"/>
+      <x:c r="F19" s="25"/>
+      <x:c r="G19" s="25"/>
+      <x:c r="H19" s="25"/>
+      <x:c r="I19" s="25"/>
       <x:c r="J19" s="1"/>
       <x:c r="K19" s="1"/>
       <x:c r="L19" s="1"/>
@@ -5728,12 +5997,12 @@
       <x:c r="A20" s="1"/>
       <x:c r="B20" s="1"/>
       <x:c r="C20" s="1"/>
-      <x:c r="D20" s="1"/>
-      <x:c r="E20" s="1"/>
-      <x:c r="F20" s="1"/>
-      <x:c r="G20" s="1"/>
-      <x:c r="H20" s="1"/>
-      <x:c r="I20" s="1"/>
+      <x:c r="D20" s="25"/>
+      <x:c r="E20" s="25"/>
+      <x:c r="F20" s="25"/>
+      <x:c r="G20" s="25"/>
+      <x:c r="H20" s="25"/>
+      <x:c r="I20" s="25"/>
       <x:c r="J20" s="1"/>
       <x:c r="K20" s="1"/>
       <x:c r="L20" s="1"/>
@@ -5741,13 +6010,30 @@
     <x:row r="21" ht="22" customHeight="1">
       <x:c r="A21" s="1"/>
       <x:c r="B21" s="1"/>
-      <x:c r="C21" s="1"/>
-      <x:c r="D21" s="1"/>
-      <x:c r="E21" s="1"/>
-      <x:c r="F21" s="1"/>
-      <x:c r="G21" s="1"/>
-      <x:c r="H21" s="1"/>
-      <x:c r="I21" s="1"/>
+      <x:c r="C21" s="1" t="str">
+        <x:v>Lease rental / fuel / downtime</x:v>
+      </x:c>
+      <x:c r="D21" s="25"/>
+      <x:c r="E21" s="26" t="n">
+        <x:f>'Cash Flows'!E26</x:f>
+        <x:v>474533.3333333333</x:v>
+      </x:c>
+      <x:c r="F21" s="26" t="n">
+        <x:f>'Cash Flows'!F26</x:f>
+        <x:v>488769.3333333333</x:v>
+      </x:c>
+      <x:c r="G21" s="26" t="n">
+        <x:f>'Cash Flows'!G26</x:f>
+        <x:v>503432.41333333333</x:v>
+      </x:c>
+      <x:c r="H21" s="26" t="n">
+        <x:f>'Cash Flows'!H26</x:f>
+        <x:v>518535.3857333333</x:v>
+      </x:c>
+      <x:c r="I21" s="26" t="n">
+        <x:f>'Cash Flows'!I26</x:f>
+        <x:v>534091.4473053333</x:v>
+      </x:c>
       <x:c r="J21" s="1"/>
       <x:c r="K21" s="1"/>
       <x:c r="L21" s="1"/>
@@ -5755,13 +6041,30 @@
     <x:row r="22" ht="22" customHeight="1">
       <x:c r="A22" s="1"/>
       <x:c r="B22" s="1"/>
-      <x:c r="C22" s="1"/>
-      <x:c r="D22" s="1"/>
-      <x:c r="E22" s="1"/>
-      <x:c r="F22" s="1"/>
-      <x:c r="G22" s="1"/>
-      <x:c r="H22" s="1"/>
-      <x:c r="I22" s="1"/>
+      <x:c r="C22" s="1" t="str">
+        <x:v>Excess mileage cost</x:v>
+      </x:c>
+      <x:c r="D22" s="25"/>
+      <x:c r="E22" s="26" t="n">
+        <x:f>MAX(0,'Assumptions'!$D$18-'Assumptions'!$I$48)*'Assumptions'!$I$49*'Assumptions'!$G$9</x:f>
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="F22" s="26" t="n">
+        <x:f>MAX(0,'Assumptions'!$D$18-'Assumptions'!$I$48)*'Assumptions'!$I$49*'Assumptions'!$G$9</x:f>
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="G22" s="26" t="n">
+        <x:f>MAX(0,'Assumptions'!$D$18-'Assumptions'!$I$48)*'Assumptions'!$I$49*'Assumptions'!$G$9</x:f>
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="H22" s="26" t="n">
+        <x:f>MAX(0,'Assumptions'!$D$18-'Assumptions'!$I$48)*'Assumptions'!$I$49*'Assumptions'!$G$9</x:f>
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="I22" s="26" t="n">
+        <x:f>MAX(0,'Assumptions'!$D$18-'Assumptions'!$I$48)*'Assumptions'!$I$49*'Assumptions'!$G$9</x:f>
+        <x:v>6000</x:v>
+      </x:c>
       <x:c r="J22" s="1"/>
       <x:c r="K22" s="1"/>
       <x:c r="L22" s="1"/>
@@ -5769,13 +6072,30 @@
     <x:row r="23" ht="22" customHeight="1">
       <x:c r="A23" s="1"/>
       <x:c r="B23" s="1"/>
-      <x:c r="C23" s="1"/>
-      <x:c r="D23" s="1"/>
-      <x:c r="E23" s="1"/>
-      <x:c r="F23" s="1"/>
-      <x:c r="G23" s="1"/>
-      <x:c r="H23" s="1"/>
-      <x:c r="I23" s="1"/>
+      <x:c r="C23" s="1" t="str">
+        <x:v>Lease tax benefit</x:v>
+      </x:c>
+      <x:c r="D23" s="25"/>
+      <x:c r="E23" s="26" t="n">
+        <x:f>SUM(E21:E22)*'Assumptions'!$I$44*'Assumptions'!$I$57</x:f>
+        <x:v>120133.33333333333</x:v>
+      </x:c>
+      <x:c r="F23" s="26" t="n">
+        <x:f>SUM(F21:F22)*'Assumptions'!$I$44*'Assumptions'!$I$57</x:f>
+        <x:v>123692.33333333333</x:v>
+      </x:c>
+      <x:c r="G23" s="26" t="n">
+        <x:f>SUM(G21:G22)*'Assumptions'!$I$44*'Assumptions'!$I$57</x:f>
+        <x:v>127358.10333333333</x:v>
+      </x:c>
+      <x:c r="H23" s="26" t="n">
+        <x:f>SUM(H21:H22)*'Assumptions'!$I$44*'Assumptions'!$I$57</x:f>
+        <x:v>131133.84643333332</x:v>
+      </x:c>
+      <x:c r="I23" s="26" t="n">
+        <x:f>SUM(I21:I22)*'Assumptions'!$I$44*'Assumptions'!$I$57</x:f>
+        <x:v>135022.86182633333</x:v>
+      </x:c>
       <x:c r="J23" s="1"/>
       <x:c r="K23" s="1"/>
       <x:c r="L23" s="1"/>
@@ -5783,13 +6103,30 @@
     <x:row r="24" ht="22" customHeight="1">
       <x:c r="A24" s="1"/>
       <x:c r="B24" s="1"/>
-      <x:c r="C24" s="1"/>
-      <x:c r="D24" s="1"/>
-      <x:c r="E24" s="1"/>
-      <x:c r="F24" s="1"/>
-      <x:c r="G24" s="1"/>
-      <x:c r="H24" s="1"/>
-      <x:c r="I24" s="1"/>
+      <x:c r="C24" s="1" t="str">
+        <x:v>Lease deposit returned</x:v>
+      </x:c>
+      <x:c r="D24" s="25"/>
+      <x:c r="E24" s="18" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F24" s="18" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G24" s="18" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H24" s="18" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I24" s="26" t="n">
+        <x:f>'Cash Flows'!I27</x:f>
+        <x:v>50000</x:v>
+      </x:c>
       <x:c r="J24" s="1"/>
       <x:c r="K24" s="1"/>
       <x:c r="L24" s="1"/>
@@ -5797,13 +6134,33 @@
     <x:row r="25" ht="22" customHeight="1">
       <x:c r="A25" s="1"/>
       <x:c r="B25" s="1"/>
-      <x:c r="C25" s="1"/>
-      <x:c r="D25" s="1"/>
-      <x:c r="E25" s="1"/>
-      <x:c r="F25" s="1"/>
-      <x:c r="G25" s="1"/>
-      <x:c r="H25" s="1"/>
-      <x:c r="I25" s="1"/>
+      <x:c r="C25" s="1" t="str">
+        <x:v>Lease unlevered cash flow</x:v>
+      </x:c>
+      <x:c r="D25" s="26" t="n">
+        <x:f>'Cash Flows'!D28-('Assumptions'!G9*('Assumptions'!G11-'Assumptions'!I45))*'Assumptions'!I44-'Assumptions'!G9*'Assumptions'!I47*(1-'Assumptions'!I44*'Assumptions'!I56*'Assumptions'!I57)</x:f>
+        <x:v>44500</x:v>
+      </x:c>
+      <x:c r="E25" s="18" t="n">
+        <x:f>-SUM(E21:E22)+SUM(E23:E24)</x:f>
+        <x:v>-360400</x:v>
+      </x:c>
+      <x:c r="F25" s="18" t="n">
+        <x:f>-SUM(F21:F22)+SUM(F23:F24)</x:f>
+        <x:v>-371077</x:v>
+      </x:c>
+      <x:c r="G25" s="18" t="n">
+        <x:f>-SUM(G21:G22)+SUM(G23:G24)</x:f>
+        <x:v>-382074.31</x:v>
+      </x:c>
+      <x:c r="H25" s="18" t="n">
+        <x:f>-SUM(H21:H22)+SUM(H23:H24)</x:f>
+        <x:v>-393401.53929999995</x:v>
+      </x:c>
+      <x:c r="I25" s="18" t="n">
+        <x:f>-SUM(I21:I22)+SUM(I23:I24)</x:f>
+        <x:v>-355068.585479</x:v>
+      </x:c>
       <x:c r="J25" s="1"/>
       <x:c r="K25" s="1"/>
       <x:c r="L25" s="1"/>
@@ -5812,12 +6169,12 @@
       <x:c r="A26" s="1"/>
       <x:c r="B26" s="1"/>
       <x:c r="C26" s="1"/>
-      <x:c r="D26" s="1"/>
-      <x:c r="E26" s="1"/>
-      <x:c r="F26" s="1"/>
-      <x:c r="G26" s="1"/>
-      <x:c r="H26" s="1"/>
-      <x:c r="I26" s="1"/>
+      <x:c r="D26" s="25"/>
+      <x:c r="E26" s="25"/>
+      <x:c r="F26" s="25"/>
+      <x:c r="G26" s="25"/>
+      <x:c r="H26" s="25"/>
+      <x:c r="I26" s="25"/>
       <x:c r="J26" s="1"/>
       <x:c r="K26" s="1"/>
       <x:c r="L26" s="1"/>
@@ -5826,12 +6183,12 @@
       <x:c r="A27" s="1"/>
       <x:c r="B27" s="1"/>
       <x:c r="C27" s="1"/>
-      <x:c r="D27" s="1"/>
-      <x:c r="E27" s="1"/>
-      <x:c r="F27" s="1"/>
-      <x:c r="G27" s="1"/>
-      <x:c r="H27" s="1"/>
-      <x:c r="I27" s="1"/>
+      <x:c r="D27" s="25"/>
+      <x:c r="E27" s="25"/>
+      <x:c r="F27" s="25"/>
+      <x:c r="G27" s="25"/>
+      <x:c r="H27" s="25"/>
+      <x:c r="I27" s="25"/>
       <x:c r="J27" s="1"/>
       <x:c r="K27" s="1"/>
       <x:c r="L27" s="1"/>
@@ -5839,13 +6196,33 @@
     <x:row r="28" ht="22" customHeight="1">
       <x:c r="A28" s="1"/>
       <x:c r="B28" s="1"/>
-      <x:c r="C28" s="1"/>
-      <x:c r="D28" s="1"/>
-      <x:c r="E28" s="1"/>
-      <x:c r="F28" s="1"/>
-      <x:c r="G28" s="1"/>
-      <x:c r="H28" s="1"/>
-      <x:c r="I28" s="1"/>
+      <x:c r="C28" s="1" t="str">
+        <x:v>Discount factor</x:v>
+      </x:c>
+      <x:c r="D28" s="27" t="n">
+        <x:f>'Cash Flows'!D34</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E28" s="27" t="n">
+        <x:f>'Cash Flows'!E34</x:f>
+        <x:v>0.9259259259259258</x:v>
+      </x:c>
+      <x:c r="F28" s="27" t="n">
+        <x:f>'Cash Flows'!F34</x:f>
+        <x:v>0.8573388203017832</x:v>
+      </x:c>
+      <x:c r="G28" s="27" t="n">
+        <x:f>'Cash Flows'!G34</x:f>
+        <x:v>0.7938322410201696</x:v>
+      </x:c>
+      <x:c r="H28" s="27" t="n">
+        <x:f>'Cash Flows'!H34</x:f>
+        <x:v>0.7350298527964533</x:v>
+      </x:c>
+      <x:c r="I28" s="27" t="n">
+        <x:f>'Cash Flows'!I34</x:f>
+        <x:v>0.6805831970337529</x:v>
+      </x:c>
       <x:c r="J28" s="1"/>
       <x:c r="K28" s="1"/>
       <x:c r="L28" s="1"/>
@@ -5853,13 +6230,33 @@
     <x:row r="29" ht="22" customHeight="1">
       <x:c r="A29" s="1"/>
       <x:c r="B29" s="1"/>
-      <x:c r="C29" s="1"/>
-      <x:c r="D29" s="1"/>
-      <x:c r="E29" s="1"/>
-      <x:c r="F29" s="1"/>
-      <x:c r="G29" s="1"/>
-      <x:c r="H29" s="1"/>
-      <x:c r="I29" s="1"/>
+      <x:c r="C29" s="1" t="str">
+        <x:v>Keep present value</x:v>
+      </x:c>
+      <x:c r="D29" s="18" t="n">
+        <x:f>D11*D28</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E29" s="18" t="n">
+        <x:f>E11*E28</x:f>
+        <x:v>-371944.4444444444</x:v>
+      </x:c>
+      <x:c r="F29" s="18" t="n">
+        <x:f>F11*F28</x:f>
+        <x:v>-354840.53497942386</x:v>
+      </x:c>
+      <x:c r="G29" s="18" t="n">
+        <x:f>G11*G28</x:f>
+        <x:v>-338519.89978661784</x:v>
+      </x:c>
+      <x:c r="H29" s="18" t="n">
+        <x:f>H11*H28</x:f>
+        <x:v>-322946.91123403155</x:v>
+      </x:c>
+      <x:c r="I29" s="18" t="n">
+        <x:f>I11*I28</x:f>
+        <x:v>-286649.17336860346</x:v>
+      </x:c>
       <x:c r="J29" s="1"/>
       <x:c r="K29" s="1"/>
       <x:c r="L29" s="1"/>
@@ -5867,13 +6264,33 @@
     <x:row r="30" ht="22" customHeight="1">
       <x:c r="A30" s="1"/>
       <x:c r="B30" s="1"/>
-      <x:c r="C30" s="1"/>
-      <x:c r="D30" s="1"/>
-      <x:c r="E30" s="1"/>
-      <x:c r="F30" s="1"/>
-      <x:c r="G30" s="1"/>
-      <x:c r="H30" s="1"/>
-      <x:c r="I30" s="1"/>
+      <x:c r="C30" s="1" t="str">
+        <x:v>Replace present value</x:v>
+      </x:c>
+      <x:c r="D30" s="18" t="n">
+        <x:f>D18*D28</x:f>
+        <x:v>-685500</x:v>
+      </x:c>
+      <x:c r="E30" s="18" t="n">
+        <x:f>E18*E28</x:f>
+        <x:v>-193425.9259259259</x:v>
+      </x:c>
+      <x:c r="F30" s="18" t="n">
+        <x:f>F18*F28</x:f>
+        <x:v>-185474.10836762688</x:v>
+      </x:c>
+      <x:c r="G30" s="18" t="n">
+        <x:f>G18*G28</x:f>
+        <x:v>-177816.12781334142</x:v>
+      </x:c>
+      <x:c r="H30" s="18" t="n">
+        <x:f>H18*H28</x:f>
+        <x:v>-170443.88460160673</x:v>
+      </x:c>
+      <x:c r="I30" s="18" t="n">
+        <x:f>I18*I28</x:f>
+        <x:v>-34719.02211934918</x:v>
+      </x:c>
       <x:c r="J30" s="1"/>
       <x:c r="K30" s="1"/>
       <x:c r="L30" s="1"/>
@@ -5881,13 +6298,33 @@
     <x:row r="31" ht="22" customHeight="1">
       <x:c r="A31" s="1"/>
       <x:c r="B31" s="1"/>
-      <x:c r="C31" s="1"/>
-      <x:c r="D31" s="1"/>
-      <x:c r="E31" s="1"/>
-      <x:c r="F31" s="1"/>
-      <x:c r="G31" s="1"/>
-      <x:c r="H31" s="1"/>
-      <x:c r="I31" s="1"/>
+      <x:c r="C31" s="1" t="str">
+        <x:v>Lease present value</x:v>
+      </x:c>
+      <x:c r="D31" s="18" t="n">
+        <x:f>D25*D28</x:f>
+        <x:v>44500</x:v>
+      </x:c>
+      <x:c r="E31" s="18" t="n">
+        <x:f>E25*E28</x:f>
+        <x:v>-333703.70370370365</x:v>
+      </x:c>
+      <x:c r="F31" s="18" t="n">
+        <x:f>F25*F28</x:f>
+        <x:v>-318138.7174211248</x:v>
+      </x:c>
+      <x:c r="G31" s="18" t="n">
+        <x:f>G25*G28</x:f>
+        <x:v>-303302.90574353497</x:v>
+      </x:c>
+      <x:c r="H31" s="18" t="n">
+        <x:f>H25*H28</x:f>
+        <x:v>-289161.8755215771</x:v>
+      </x:c>
+      <x:c r="I31" s="18" t="n">
+        <x:f>I25*I28</x:f>
+        <x:v>-241653.71307155018</x:v>
+      </x:c>
       <x:c r="J31" s="1"/>
       <x:c r="K31" s="1"/>
       <x:c r="L31" s="1"/>
@@ -5896,12 +6333,12 @@
       <x:c r="A32" s="1"/>
       <x:c r="B32" s="1"/>
       <x:c r="C32" s="1"/>
-      <x:c r="D32" s="1"/>
-      <x:c r="E32" s="1"/>
-      <x:c r="F32" s="1"/>
-      <x:c r="G32" s="1"/>
-      <x:c r="H32" s="1"/>
-      <x:c r="I32" s="1"/>
+      <x:c r="D32" s="25"/>
+      <x:c r="E32" s="25"/>
+      <x:c r="F32" s="25"/>
+      <x:c r="G32" s="25"/>
+      <x:c r="H32" s="25"/>
+      <x:c r="I32" s="25"/>
       <x:c r="J32" s="1"/>
       <x:c r="K32" s="1"/>
       <x:c r="L32" s="1"/>
@@ -5910,12 +6347,12 @@
       <x:c r="A33" s="1"/>
       <x:c r="B33" s="1"/>
       <x:c r="C33" s="1"/>
-      <x:c r="D33" s="1"/>
-      <x:c r="E33" s="1"/>
-      <x:c r="F33" s="1"/>
-      <x:c r="G33" s="1"/>
-      <x:c r="H33" s="1"/>
-      <x:c r="I33" s="1"/>
+      <x:c r="D33" s="25"/>
+      <x:c r="E33" s="25"/>
+      <x:c r="F33" s="25"/>
+      <x:c r="G33" s="25"/>
+      <x:c r="H33" s="25"/>
+      <x:c r="I33" s="25"/>
       <x:c r="J33" s="1"/>
       <x:c r="K33" s="1"/>
       <x:c r="L33" s="1"/>
@@ -5923,13 +6360,33 @@
     <x:row r="34" ht="22" customHeight="1">
       <x:c r="A34" s="1"/>
       <x:c r="B34" s="1"/>
-      <x:c r="C34" s="1"/>
-      <x:c r="D34" s="1"/>
-      <x:c r="E34" s="1"/>
-      <x:c r="F34" s="1"/>
-      <x:c r="G34" s="1"/>
-      <x:c r="H34" s="1"/>
-      <x:c r="I34" s="1"/>
+      <x:c r="C34" s="1" t="str">
+        <x:v>Replacement vs keep cash flow</x:v>
+      </x:c>
+      <x:c r="D34" s="18" t="n">
+        <x:f>D18-D11</x:f>
+        <x:v>-685500</x:v>
+      </x:c>
+      <x:c r="E34" s="18" t="n">
+        <x:f>E18-E11</x:f>
+        <x:v>192800</x:v>
+      </x:c>
+      <x:c r="F34" s="18" t="n">
+        <x:f>F18-F11</x:f>
+        <x:v>197549</x:v>
+      </x:c>
+      <x:c r="G34" s="18" t="n">
+        <x:f>G18-G11</x:f>
+        <x:v>202440.46999999997</x:v>
+      </x:c>
+      <x:c r="H34" s="18" t="n">
+        <x:f>H18-H11</x:f>
+        <x:v>207478.68409999995</x:v>
+      </x:c>
+      <x:c r="I34" s="18" t="n">
+        <x:f>I18-I11</x:f>
+        <x:v>370168.044623</x:v>
+      </x:c>
       <x:c r="J34" s="1"/>
       <x:c r="K34" s="1"/>
       <x:c r="L34" s="1"/>
@@ -5937,13 +6394,33 @@
     <x:row r="35" ht="22" customHeight="1">
       <x:c r="A35" s="1"/>
       <x:c r="B35" s="1"/>
-      <x:c r="C35" s="1"/>
-      <x:c r="D35" s="1"/>
-      <x:c r="E35" s="1"/>
-      <x:c r="F35" s="1"/>
-      <x:c r="G35" s="1"/>
-      <x:c r="H35" s="1"/>
-      <x:c r="I35" s="1"/>
+      <x:c r="C35" s="1" t="str">
+        <x:v>Lease vs keep cash flow</x:v>
+      </x:c>
+      <x:c r="D35" s="18" t="n">
+        <x:f>D25-D11</x:f>
+        <x:v>44500</x:v>
+      </x:c>
+      <x:c r="E35" s="18" t="n">
+        <x:f>E25-E11</x:f>
+        <x:v>41300</x:v>
+      </x:c>
+      <x:c r="F35" s="18" t="n">
+        <x:f>F25-F11</x:f>
+        <x:v>42809</x:v>
+      </x:c>
+      <x:c r="G35" s="18" t="n">
+        <x:f>G25-G11</x:f>
+        <x:v>44363.26999999996</x:v>
+      </x:c>
+      <x:c r="H35" s="18" t="n">
+        <x:f>H25-H11</x:f>
+        <x:v>45964.16810000001</x:v>
+      </x:c>
+      <x:c r="I35" s="18" t="n">
+        <x:f>I25-I11</x:f>
+        <x:v>66113.09314300003</x:v>
+      </x:c>
       <x:c r="J35" s="1"/>
       <x:c r="K35" s="1"/>
       <x:c r="L35" s="1"/>
@@ -6370,13 +6847,8 @@
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="C4:I4"/>
+    <x:mergeCell ref="D4:F4"/>
   </x:mergeCells>
-  <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="H7:H10">
-      <x:formula1>"Proposed,In progress,Completed,Blocked"</x:formula1>
-    </x:dataValidation>
-  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -6417,7 +6889,7 @@
       <x:c r="A2" s="1"/>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="2" t="str">
-        <x:v>Reconciliation checks</x:v>
+        <x:v>Purchase financing and lease obligations</x:v>
       </x:c>
       <x:c r="D2" s="1"/>
       <x:c r="E2" s="1"/>
@@ -6446,8 +6918,13 @@
     <x:row r="4" ht="22" customHeight="1">
       <x:c r="A4" s="1"/>
       <x:c r="B4" s="1"/>
-      <x:c r="C4" s="1"/>
-      <x:c r="D4" s="1"/>
+      <x:c r="C4" s="1" t="str">
+        <x:v>Case selected</x:v>
+      </x:c>
+      <x:c r="D4" s="7" t="str">
+        <x:f>'Assumptions'!D4</x:f>
+        <x:v>Base</x:v>
+      </x:c>
       <x:c r="E4" s="1"/>
       <x:c r="F4" s="1"/>
       <x:c r="G4" s="1"/>
@@ -6471,6 +6948,2206 @@
       <x:c r="K5" s="1"/>
       <x:c r="L5" s="1"/>
     </x:row>
+    <x:row r="6" ht="22" customHeight="1">
+      <x:c r="A6" s="1"/>
+      <x:c r="B6" s="1"/>
+      <x:c r="C6" s="1"/>
+      <x:c r="D6" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E6" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F6" s="4" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G6" s="4" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H6" s="4" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I6" s="4" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J6" s="1"/>
+      <x:c r="K6" s="1"/>
+      <x:c r="L6" s="1"/>
+    </x:row>
+    <x:row r="7" ht="22" customHeight="1">
+      <x:c r="A7" s="1"/>
+      <x:c r="B7" s="1"/>
+      <x:c r="C7" s="1" t="str">
+        <x:v>Opening purchase loan</x:v>
+      </x:c>
+      <x:c r="D7" s="18" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E7" s="26" t="n">
+        <x:f>'Assumptions'!G9*'Assumptions'!G10*'Assumptions'!I50</x:f>
+        <x:v>546000</x:v>
+      </x:c>
+      <x:c r="F7" s="18" t="n">
+        <x:f>E10</x:f>
+        <x:v>436800</x:v>
+      </x:c>
+      <x:c r="G7" s="18" t="n">
+        <x:f>F10</x:f>
+        <x:v>327600</x:v>
+      </x:c>
+      <x:c r="H7" s="18" t="n">
+        <x:f>G10</x:f>
+        <x:v>218400</x:v>
+      </x:c>
+      <x:c r="I7" s="18" t="n">
+        <x:f>H10</x:f>
+        <x:v>109200</x:v>
+      </x:c>
+      <x:c r="J7" s="1"/>
+      <x:c r="K7" s="1"/>
+      <x:c r="L7" s="1"/>
+    </x:row>
+    <x:row r="8" ht="22" customHeight="1">
+      <x:c r="A8" s="1"/>
+      <x:c r="B8" s="1"/>
+      <x:c r="C8" s="1" t="str">
+        <x:v>Loan draw</x:v>
+      </x:c>
+      <x:c r="D8" s="26" t="n">
+        <x:f>'Assumptions'!G9*'Assumptions'!G10*'Assumptions'!I50</x:f>
+        <x:v>546000</x:v>
+      </x:c>
+      <x:c r="E8" s="18" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F8" s="18" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G8" s="18" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H8" s="18" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I8" s="18" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J8" s="1"/>
+      <x:c r="K8" s="1"/>
+      <x:c r="L8" s="1"/>
+    </x:row>
+    <x:row r="9" ht="22" customHeight="1">
+      <x:c r="A9" s="1"/>
+      <x:c r="B9" s="1"/>
+      <x:c r="C9" s="1" t="str">
+        <x:v>Principal repayment</x:v>
+      </x:c>
+      <x:c r="D9" s="18" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E9" s="18" t="n">
+        <x:f>MIN(E7,$D$8/5)</x:f>
+        <x:v>109200</x:v>
+      </x:c>
+      <x:c r="F9" s="18" t="n">
+        <x:f>MIN(F7,$D$8/5)</x:f>
+        <x:v>109200</x:v>
+      </x:c>
+      <x:c r="G9" s="18" t="n">
+        <x:f>MIN(G7,$D$8/5)</x:f>
+        <x:v>109200</x:v>
+      </x:c>
+      <x:c r="H9" s="18" t="n">
+        <x:f>MIN(H7,$D$8/5)</x:f>
+        <x:v>109200</x:v>
+      </x:c>
+      <x:c r="I9" s="18" t="n">
+        <x:f>MIN(I7,$D$8/5)</x:f>
+        <x:v>109200</x:v>
+      </x:c>
+      <x:c r="J9" s="1"/>
+      <x:c r="K9" s="1"/>
+      <x:c r="L9" s="1"/>
+    </x:row>
+    <x:row r="10" ht="22" customHeight="1">
+      <x:c r="A10" s="1"/>
+      <x:c r="B10" s="1"/>
+      <x:c r="C10" s="1" t="str">
+        <x:v>Closing purchase loan</x:v>
+      </x:c>
+      <x:c r="D10" s="18" t="n">
+        <x:f>SUM(D7:D8)-D9</x:f>
+        <x:v>546000</x:v>
+      </x:c>
+      <x:c r="E10" s="18" t="n">
+        <x:f>SUM(E7:E8)-E9</x:f>
+        <x:v>436800</x:v>
+      </x:c>
+      <x:c r="F10" s="18" t="n">
+        <x:f>SUM(F7:F8)-F9</x:f>
+        <x:v>327600</x:v>
+      </x:c>
+      <x:c r="G10" s="18" t="n">
+        <x:f>SUM(G7:G8)-G9</x:f>
+        <x:v>218400</x:v>
+      </x:c>
+      <x:c r="H10" s="18" t="n">
+        <x:f>SUM(H7:H8)-H9</x:f>
+        <x:v>109200</x:v>
+      </x:c>
+      <x:c r="I10" s="18" t="n">
+        <x:f>SUM(I7:I8)-I9</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J10" s="1"/>
+      <x:c r="K10" s="1"/>
+      <x:c r="L10" s="1"/>
+    </x:row>
+    <x:row r="11" ht="22" customHeight="1">
+      <x:c r="A11" s="1"/>
+      <x:c r="B11" s="1"/>
+      <x:c r="C11" s="1" t="str">
+        <x:v>Cash interest</x:v>
+      </x:c>
+      <x:c r="D11" s="18" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E11" s="26" t="n">
+        <x:f>E7*'Assumptions'!$I$51</x:f>
+        <x:v>40950</x:v>
+      </x:c>
+      <x:c r="F11" s="26" t="n">
+        <x:f>F7*'Assumptions'!$I$51</x:f>
+        <x:v>32760</x:v>
+      </x:c>
+      <x:c r="G11" s="26" t="n">
+        <x:f>G7*'Assumptions'!$I$51</x:f>
+        <x:v>24570</x:v>
+      </x:c>
+      <x:c r="H11" s="26" t="n">
+        <x:f>H7*'Assumptions'!$I$51</x:f>
+        <x:v>16380</x:v>
+      </x:c>
+      <x:c r="I11" s="26" t="n">
+        <x:f>I7*'Assumptions'!$I$51</x:f>
+        <x:v>8190</x:v>
+      </x:c>
+      <x:c r="J11" s="1"/>
+      <x:c r="K11" s="1"/>
+      <x:c r="L11" s="1"/>
+    </x:row>
+    <x:row r="12" ht="22" customHeight="1">
+      <x:c r="A12" s="1"/>
+      <x:c r="B12" s="1"/>
+      <x:c r="C12" s="1" t="str">
+        <x:v>Origination fee</x:v>
+      </x:c>
+      <x:c r="D12" s="26" t="n">
+        <x:f>D8*'Assumptions'!I52</x:f>
+        <x:v>5460</x:v>
+      </x:c>
+      <x:c r="E12" s="18" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F12" s="18" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G12" s="18" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H12" s="18" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I12" s="18" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J12" s="1"/>
+      <x:c r="K12" s="1"/>
+      <x:c r="L12" s="1"/>
+    </x:row>
+    <x:row r="13" ht="22" customHeight="1">
+      <x:c r="A13" s="1"/>
+      <x:c r="B13" s="1"/>
+      <x:c r="C13" s="1" t="str">
+        <x:v>Interest tax benefit</x:v>
+      </x:c>
+      <x:c r="D13" s="26" t="n">
+        <x:f>D11*'Assumptions'!$I$44*'Assumptions'!$I$57</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E13" s="26" t="n">
+        <x:f>E11*'Assumptions'!$I$44*'Assumptions'!$I$57</x:f>
+        <x:v>10237.5</x:v>
+      </x:c>
+      <x:c r="F13" s="26" t="n">
+        <x:f>F11*'Assumptions'!$I$44*'Assumptions'!$I$57</x:f>
+        <x:v>8190</x:v>
+      </x:c>
+      <x:c r="G13" s="26" t="n">
+        <x:f>G11*'Assumptions'!$I$44*'Assumptions'!$I$57</x:f>
+        <x:v>6142.5</x:v>
+      </x:c>
+      <x:c r="H13" s="26" t="n">
+        <x:f>H11*'Assumptions'!$I$44*'Assumptions'!$I$57</x:f>
+        <x:v>4095</x:v>
+      </x:c>
+      <x:c r="I13" s="26" t="n">
+        <x:f>I11*'Assumptions'!$I$44*'Assumptions'!$I$57</x:f>
+        <x:v>2047.5</x:v>
+      </x:c>
+      <x:c r="J13" s="1"/>
+      <x:c r="K13" s="1"/>
+      <x:c r="L13" s="1"/>
+    </x:row>
+    <x:row r="14" ht="22" customHeight="1">
+      <x:c r="A14" s="1"/>
+      <x:c r="B14" s="1"/>
+      <x:c r="C14" s="1" t="str">
+        <x:v>Replace equity cash flow</x:v>
+      </x:c>
+      <x:c r="D14" s="26" t="n">
+        <x:f>'After Tax'!D18+D8-D9-D11-D12+D13</x:f>
+        <x:v>-144960</x:v>
+      </x:c>
+      <x:c r="E14" s="26" t="n">
+        <x:f>'After Tax'!E18+E8-E9-E11-E12+E13</x:f>
+        <x:v>-348812.5</x:v>
+      </x:c>
+      <x:c r="F14" s="26" t="n">
+        <x:f>'After Tax'!F18+F8-F9-F11-F12+F13</x:f>
+        <x:v>-350107</x:v>
+      </x:c>
+      <x:c r="G14" s="26" t="n">
+        <x:f>'After Tax'!G18+G8-G9-G11-G12+G13</x:f>
+        <x:v>-351624.61</x:v>
+      </x:c>
+      <x:c r="H14" s="26" t="n">
+        <x:f>'After Tax'!H18+H8-H9-H11-H12+H13</x:f>
+        <x:v>-353372.0233</x:v>
+      </x:c>
+      <x:c r="I14" s="26" t="n">
+        <x:f>'After Tax'!I18+I8-I9-I11-I12+I13</x:f>
+        <x:v>-166356.133999</x:v>
+      </x:c>
+      <x:c r="J14" s="1"/>
+      <x:c r="K14" s="1"/>
+      <x:c r="L14" s="1"/>
+    </x:row>
+    <x:row r="15" ht="22" customHeight="1">
+      <x:c r="A15" s="1"/>
+      <x:c r="B15" s="1"/>
+      <x:c r="C15" s="1"/>
+      <x:c r="D15" s="25"/>
+      <x:c r="E15" s="25"/>
+      <x:c r="F15" s="25"/>
+      <x:c r="G15" s="25"/>
+      <x:c r="H15" s="25"/>
+      <x:c r="I15" s="25"/>
+      <x:c r="J15" s="1"/>
+      <x:c r="K15" s="1"/>
+      <x:c r="L15" s="1"/>
+    </x:row>
+    <x:row r="16" ht="22" customHeight="1">
+      <x:c r="A16" s="1"/>
+      <x:c r="B16" s="1"/>
+      <x:c r="C16" s="1"/>
+      <x:c r="D16" s="25"/>
+      <x:c r="E16" s="25"/>
+      <x:c r="F16" s="25"/>
+      <x:c r="G16" s="25"/>
+      <x:c r="H16" s="25"/>
+      <x:c r="I16" s="25"/>
+      <x:c r="J16" s="1"/>
+      <x:c r="K16" s="1"/>
+      <x:c r="L16" s="1"/>
+    </x:row>
+    <x:row r="17" ht="22" customHeight="1">
+      <x:c r="A17" s="1"/>
+      <x:c r="B17" s="1"/>
+      <x:c r="C17" s="1" t="str">
+        <x:v>Opening lease liability</x:v>
+      </x:c>
+      <x:c r="D17" s="26" t="n">
+        <x:f>NPV('Assumptions'!I53,'Cash Flows'!E23:I23)</x:f>
+        <x:v>846989.5996612386</x:v>
+      </x:c>
+      <x:c r="E17" s="18" t="n">
+        <x:f>D20</x:f>
+        <x:v>846989.5996612386</x:v>
+      </x:c>
+      <x:c r="F17" s="18" t="n">
+        <x:f>E20</x:f>
+        <x:v>712513.8196358315</x:v>
+      </x:c>
+      <x:c r="G17" s="18" t="n">
+        <x:f>F20</x:f>
+        <x:v>562012.3561085189</x:v>
+      </x:c>
+      <x:c r="H17" s="18" t="n">
+        <x:f>G20</x:f>
+        <x:v>394105.08281665784</x:v>
+      </x:c>
+      <x:c r="I17" s="18" t="n">
+        <x:f>H20</x:f>
+        <x:v>207303.01802790718</x:v>
+      </x:c>
+      <x:c r="J17" s="1"/>
+      <x:c r="K17" s="1"/>
+      <x:c r="L17" s="1"/>
+    </x:row>
+    <x:row r="18" ht="22" customHeight="1">
+      <x:c r="A18" s="1"/>
+      <x:c r="B18" s="1"/>
+      <x:c r="C18" s="1" t="str">
+        <x:v>Lease liability interest</x:v>
+      </x:c>
+      <x:c r="D18" s="18" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E18" s="26" t="n">
+        <x:f>E17*'Assumptions'!$I$53</x:f>
+        <x:v>63524.219974592896</x:v>
+      </x:c>
+      <x:c r="F18" s="26" t="n">
+        <x:f>F17*'Assumptions'!$I$53</x:f>
+        <x:v>53438.53647268736</x:v>
+      </x:c>
+      <x:c r="G18" s="26" t="n">
+        <x:f>G17*'Assumptions'!$I$53</x:f>
+        <x:v>42150.92670813892</x:v>
+      </x:c>
+      <x:c r="H18" s="26" t="n">
+        <x:f>H17*'Assumptions'!$I$53</x:f>
+        <x:v>29557.881211249336</x:v>
+      </x:c>
+      <x:c r="I18" s="26" t="n">
+        <x:f>I17*'Assumptions'!$I$53</x:f>
+        <x:v>15547.726352093037</x:v>
+      </x:c>
+      <x:c r="J18" s="1"/>
+      <x:c r="K18" s="1"/>
+      <x:c r="L18" s="1"/>
+    </x:row>
+    <x:row r="19" ht="22" customHeight="1">
+      <x:c r="A19" s="1"/>
+      <x:c r="B19" s="1"/>
+      <x:c r="C19" s="1" t="str">
+        <x:v>Contract rental payment</x:v>
+      </x:c>
+      <x:c r="D19" s="18" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E19" s="26" t="n">
+        <x:f>'Cash Flows'!E23</x:f>
+        <x:v>198000</x:v>
+      </x:c>
+      <x:c r="F19" s="26" t="n">
+        <x:f>'Cash Flows'!F23</x:f>
+        <x:v>203940</x:v>
+      </x:c>
+      <x:c r="G19" s="26" t="n">
+        <x:f>'Cash Flows'!G23</x:f>
+        <x:v>210058.19999999998</x:v>
+      </x:c>
+      <x:c r="H19" s="26" t="n">
+        <x:f>'Cash Flows'!H23</x:f>
+        <x:v>216359.946</x:v>
+      </x:c>
+      <x:c r="I19" s="26" t="n">
+        <x:f>'Cash Flows'!I23</x:f>
+        <x:v>222850.74438000002</x:v>
+      </x:c>
+      <x:c r="J19" s="1"/>
+      <x:c r="K19" s="1"/>
+      <x:c r="L19" s="1"/>
+    </x:row>
+    <x:row r="20" ht="22" customHeight="1">
+      <x:c r="A20" s="1"/>
+      <x:c r="B20" s="1"/>
+      <x:c r="C20" s="1" t="str">
+        <x:v>Closing lease liability</x:v>
+      </x:c>
+      <x:c r="D20" s="18" t="n">
+        <x:f>D17</x:f>
+        <x:v>846989.5996612386</x:v>
+      </x:c>
+      <x:c r="E20" s="18" t="n">
+        <x:f>SUM(E17:E18)-E19</x:f>
+        <x:v>712513.8196358315</x:v>
+      </x:c>
+      <x:c r="F20" s="18" t="n">
+        <x:f>SUM(F17:F18)-F19</x:f>
+        <x:v>562012.3561085189</x:v>
+      </x:c>
+      <x:c r="G20" s="18" t="n">
+        <x:f>SUM(G17:G18)-G19</x:f>
+        <x:v>394105.08281665784</x:v>
+      </x:c>
+      <x:c r="H20" s="18" t="n">
+        <x:f>SUM(H17:H18)-H19</x:f>
+        <x:v>207303.01802790718</x:v>
+      </x:c>
+      <x:c r="I20" s="18" t="n">
+        <x:f>SUM(I17:I18)-I19</x:f>
+        <x:v>2.0372681319713593e-10</x:v>
+      </x:c>
+      <x:c r="J20" s="1"/>
+      <x:c r="K20" s="1"/>
+      <x:c r="L20" s="1"/>
+    </x:row>
+    <x:row r="21" ht="22" customHeight="1">
+      <x:c r="A21" s="1"/>
+      <x:c r="B21" s="1"/>
+      <x:c r="C21" s="1"/>
+      <x:c r="D21" s="1"/>
+      <x:c r="E21" s="1"/>
+      <x:c r="F21" s="1"/>
+      <x:c r="G21" s="1"/>
+      <x:c r="H21" s="1"/>
+      <x:c r="I21" s="1"/>
+      <x:c r="J21" s="1"/>
+      <x:c r="K21" s="1"/>
+      <x:c r="L21" s="1"/>
+    </x:row>
+    <x:row r="22" ht="22" customHeight="1">
+      <x:c r="A22" s="1"/>
+      <x:c r="B22" s="1"/>
+      <x:c r="C22" s="1"/>
+      <x:c r="D22" s="1"/>
+      <x:c r="E22" s="1"/>
+      <x:c r="F22" s="1"/>
+      <x:c r="G22" s="1"/>
+      <x:c r="H22" s="1"/>
+      <x:c r="I22" s="1"/>
+      <x:c r="J22" s="1"/>
+      <x:c r="K22" s="1"/>
+      <x:c r="L22" s="1"/>
+    </x:row>
+    <x:row r="23" ht="22" customHeight="1">
+      <x:c r="A23" s="1"/>
+      <x:c r="B23" s="1"/>
+      <x:c r="C23" s="1"/>
+      <x:c r="D23" s="1"/>
+      <x:c r="E23" s="1"/>
+      <x:c r="F23" s="1"/>
+      <x:c r="G23" s="1"/>
+      <x:c r="H23" s="1"/>
+      <x:c r="I23" s="1"/>
+      <x:c r="J23" s="1"/>
+      <x:c r="K23" s="1"/>
+      <x:c r="L23" s="1"/>
+    </x:row>
+    <x:row r="24" ht="22" customHeight="1">
+      <x:c r="A24" s="1"/>
+      <x:c r="B24" s="1"/>
+      <x:c r="C24" s="5" t="str">
+        <x:v>Loan cash flows are separate from unlevered NPV. Lease liability is a simplified obligation roll-forward.</x:v>
+      </x:c>
+      <x:c r="D24" s="5"/>
+      <x:c r="E24" s="5"/>
+      <x:c r="F24" s="5"/>
+      <x:c r="G24" s="5"/>
+      <x:c r="H24" s="5"/>
+      <x:c r="I24" s="5"/>
+      <x:c r="J24" s="5"/>
+      <x:c r="K24" s="5"/>
+      <x:c r="L24" s="1"/>
+    </x:row>
+    <x:row r="25" ht="22" customHeight="1">
+      <x:c r="A25" s="1"/>
+      <x:c r="B25" s="1"/>
+      <x:c r="C25" s="5"/>
+      <x:c r="D25" s="5"/>
+      <x:c r="E25" s="5"/>
+      <x:c r="F25" s="5"/>
+      <x:c r="G25" s="5"/>
+      <x:c r="H25" s="5"/>
+      <x:c r="I25" s="5"/>
+      <x:c r="J25" s="5"/>
+      <x:c r="K25" s="5"/>
+      <x:c r="L25" s="1"/>
+    </x:row>
+    <x:row r="26" ht="22" customHeight="1">
+      <x:c r="A26" s="1"/>
+      <x:c r="B26" s="1"/>
+      <x:c r="C26" s="5"/>
+      <x:c r="D26" s="5"/>
+      <x:c r="E26" s="5"/>
+      <x:c r="F26" s="5"/>
+      <x:c r="G26" s="5"/>
+      <x:c r="H26" s="5"/>
+      <x:c r="I26" s="5"/>
+      <x:c r="J26" s="5"/>
+      <x:c r="K26" s="5"/>
+      <x:c r="L26" s="1"/>
+    </x:row>
+    <x:row r="27" ht="22" customHeight="1">
+      <x:c r="A27" s="1"/>
+      <x:c r="B27" s="1"/>
+      <x:c r="C27" s="1"/>
+      <x:c r="D27" s="1"/>
+      <x:c r="E27" s="1"/>
+      <x:c r="F27" s="1"/>
+      <x:c r="G27" s="1"/>
+      <x:c r="H27" s="1"/>
+      <x:c r="I27" s="1"/>
+      <x:c r="J27" s="1"/>
+      <x:c r="K27" s="1"/>
+      <x:c r="L27" s="1"/>
+    </x:row>
+    <x:row r="28" ht="22" customHeight="1">
+      <x:c r="A28" s="1"/>
+      <x:c r="B28" s="1"/>
+      <x:c r="C28" s="1"/>
+      <x:c r="D28" s="1"/>
+      <x:c r="E28" s="1"/>
+      <x:c r="F28" s="1"/>
+      <x:c r="G28" s="1"/>
+      <x:c r="H28" s="1"/>
+      <x:c r="I28" s="1"/>
+      <x:c r="J28" s="1"/>
+      <x:c r="K28" s="1"/>
+      <x:c r="L28" s="1"/>
+    </x:row>
+    <x:row r="29" ht="22" customHeight="1">
+      <x:c r="A29" s="1"/>
+      <x:c r="B29" s="1"/>
+      <x:c r="C29" s="1"/>
+      <x:c r="D29" s="1"/>
+      <x:c r="E29" s="1"/>
+      <x:c r="F29" s="1"/>
+      <x:c r="G29" s="1"/>
+      <x:c r="H29" s="1"/>
+      <x:c r="I29" s="1"/>
+      <x:c r="J29" s="1"/>
+      <x:c r="K29" s="1"/>
+      <x:c r="L29" s="1"/>
+    </x:row>
+    <x:row r="30" ht="22" customHeight="1">
+      <x:c r="A30" s="1"/>
+      <x:c r="B30" s="1"/>
+      <x:c r="C30" s="1"/>
+      <x:c r="D30" s="1"/>
+      <x:c r="E30" s="1"/>
+      <x:c r="F30" s="1"/>
+      <x:c r="G30" s="1"/>
+      <x:c r="H30" s="1"/>
+      <x:c r="I30" s="1"/>
+      <x:c r="J30" s="1"/>
+      <x:c r="K30" s="1"/>
+      <x:c r="L30" s="1"/>
+    </x:row>
+    <x:row r="31" ht="22" customHeight="1">
+      <x:c r="A31" s="1"/>
+      <x:c r="B31" s="1"/>
+      <x:c r="C31" s="1"/>
+      <x:c r="D31" s="1"/>
+      <x:c r="E31" s="1"/>
+      <x:c r="F31" s="1"/>
+      <x:c r="G31" s="1"/>
+      <x:c r="H31" s="1"/>
+      <x:c r="I31" s="1"/>
+      <x:c r="J31" s="1"/>
+      <x:c r="K31" s="1"/>
+      <x:c r="L31" s="1"/>
+    </x:row>
+    <x:row r="32" ht="22" customHeight="1">
+      <x:c r="A32" s="1"/>
+      <x:c r="B32" s="1"/>
+      <x:c r="C32" s="1"/>
+      <x:c r="D32" s="1"/>
+      <x:c r="E32" s="1"/>
+      <x:c r="F32" s="1"/>
+      <x:c r="G32" s="1"/>
+      <x:c r="H32" s="1"/>
+      <x:c r="I32" s="1"/>
+      <x:c r="J32" s="1"/>
+      <x:c r="K32" s="1"/>
+      <x:c r="L32" s="1"/>
+    </x:row>
+    <x:row r="33" ht="22" customHeight="1">
+      <x:c r="A33" s="1"/>
+      <x:c r="B33" s="1"/>
+      <x:c r="C33" s="1"/>
+      <x:c r="D33" s="1"/>
+      <x:c r="E33" s="1"/>
+      <x:c r="F33" s="1"/>
+      <x:c r="G33" s="1"/>
+      <x:c r="H33" s="1"/>
+      <x:c r="I33" s="1"/>
+      <x:c r="J33" s="1"/>
+      <x:c r="K33" s="1"/>
+      <x:c r="L33" s="1"/>
+    </x:row>
+    <x:row r="34" ht="22" customHeight="1">
+      <x:c r="A34" s="1"/>
+      <x:c r="B34" s="1"/>
+      <x:c r="C34" s="1"/>
+      <x:c r="D34" s="1"/>
+      <x:c r="E34" s="1"/>
+      <x:c r="F34" s="1"/>
+      <x:c r="G34" s="1"/>
+      <x:c r="H34" s="1"/>
+      <x:c r="I34" s="1"/>
+      <x:c r="J34" s="1"/>
+      <x:c r="K34" s="1"/>
+      <x:c r="L34" s="1"/>
+    </x:row>
+    <x:row r="35" ht="22" customHeight="1">
+      <x:c r="A35" s="1"/>
+      <x:c r="B35" s="1"/>
+      <x:c r="C35" s="1"/>
+      <x:c r="D35" s="1"/>
+      <x:c r="E35" s="1"/>
+      <x:c r="F35" s="1"/>
+      <x:c r="G35" s="1"/>
+      <x:c r="H35" s="1"/>
+      <x:c r="I35" s="1"/>
+      <x:c r="J35" s="1"/>
+      <x:c r="K35" s="1"/>
+      <x:c r="L35" s="1"/>
+    </x:row>
+    <x:row r="36" ht="22" customHeight="1">
+      <x:c r="A36" s="1"/>
+      <x:c r="B36" s="1"/>
+      <x:c r="C36" s="1"/>
+      <x:c r="D36" s="1"/>
+      <x:c r="E36" s="1"/>
+      <x:c r="F36" s="1"/>
+      <x:c r="G36" s="1"/>
+      <x:c r="H36" s="1"/>
+      <x:c r="I36" s="1"/>
+      <x:c r="J36" s="1"/>
+      <x:c r="K36" s="1"/>
+      <x:c r="L36" s="1"/>
+    </x:row>
+    <x:row r="37" ht="22" customHeight="1">
+      <x:c r="A37" s="1"/>
+      <x:c r="B37" s="1"/>
+      <x:c r="C37" s="1"/>
+      <x:c r="D37" s="1"/>
+      <x:c r="E37" s="1"/>
+      <x:c r="F37" s="1"/>
+      <x:c r="G37" s="1"/>
+      <x:c r="H37" s="1"/>
+      <x:c r="I37" s="1"/>
+      <x:c r="J37" s="1"/>
+      <x:c r="K37" s="1"/>
+      <x:c r="L37" s="1"/>
+    </x:row>
+    <x:row r="38" ht="22" customHeight="1">
+      <x:c r="A38" s="1"/>
+      <x:c r="B38" s="1"/>
+      <x:c r="C38" s="1"/>
+      <x:c r="D38" s="1"/>
+      <x:c r="E38" s="1"/>
+      <x:c r="F38" s="1"/>
+      <x:c r="G38" s="1"/>
+      <x:c r="H38" s="1"/>
+      <x:c r="I38" s="1"/>
+      <x:c r="J38" s="1"/>
+      <x:c r="K38" s="1"/>
+      <x:c r="L38" s="1"/>
+    </x:row>
+    <x:row r="39" ht="22" customHeight="1">
+      <x:c r="A39" s="1"/>
+      <x:c r="B39" s="1"/>
+      <x:c r="C39" s="1"/>
+      <x:c r="D39" s="1"/>
+      <x:c r="E39" s="1"/>
+      <x:c r="F39" s="1"/>
+      <x:c r="G39" s="1"/>
+      <x:c r="H39" s="1"/>
+      <x:c r="I39" s="1"/>
+      <x:c r="J39" s="1"/>
+      <x:c r="K39" s="1"/>
+      <x:c r="L39" s="1"/>
+    </x:row>
+    <x:row r="40" ht="22" customHeight="1">
+      <x:c r="A40" s="1"/>
+      <x:c r="B40" s="1"/>
+      <x:c r="C40" s="1"/>
+      <x:c r="D40" s="1"/>
+      <x:c r="E40" s="1"/>
+      <x:c r="F40" s="1"/>
+      <x:c r="G40" s="1"/>
+      <x:c r="H40" s="1"/>
+      <x:c r="I40" s="1"/>
+      <x:c r="J40" s="1"/>
+      <x:c r="K40" s="1"/>
+      <x:c r="L40" s="1"/>
+    </x:row>
+    <x:row r="41" ht="22" customHeight="1">
+      <x:c r="A41" s="1"/>
+      <x:c r="B41" s="1"/>
+      <x:c r="C41" s="1"/>
+      <x:c r="D41" s="1"/>
+      <x:c r="E41" s="1"/>
+      <x:c r="F41" s="1"/>
+      <x:c r="G41" s="1"/>
+      <x:c r="H41" s="1"/>
+      <x:c r="I41" s="1"/>
+      <x:c r="J41" s="1"/>
+      <x:c r="K41" s="1"/>
+      <x:c r="L41" s="1"/>
+    </x:row>
+    <x:row r="42" ht="22" customHeight="1">
+      <x:c r="A42" s="1"/>
+      <x:c r="B42" s="1"/>
+      <x:c r="C42" s="1"/>
+      <x:c r="D42" s="1"/>
+      <x:c r="E42" s="1"/>
+      <x:c r="F42" s="1"/>
+      <x:c r="G42" s="1"/>
+      <x:c r="H42" s="1"/>
+      <x:c r="I42" s="1"/>
+      <x:c r="J42" s="1"/>
+      <x:c r="K42" s="1"/>
+      <x:c r="L42" s="1"/>
+    </x:row>
+    <x:row r="43" ht="22" customHeight="1">
+      <x:c r="A43" s="1"/>
+      <x:c r="B43" s="1"/>
+      <x:c r="C43" s="1"/>
+      <x:c r="D43" s="1"/>
+      <x:c r="E43" s="1"/>
+      <x:c r="F43" s="1"/>
+      <x:c r="G43" s="1"/>
+      <x:c r="H43" s="1"/>
+      <x:c r="I43" s="1"/>
+      <x:c r="J43" s="1"/>
+      <x:c r="K43" s="1"/>
+      <x:c r="L43" s="1"/>
+    </x:row>
+    <x:row r="44" ht="22" customHeight="1">
+      <x:c r="A44" s="1"/>
+      <x:c r="B44" s="1"/>
+      <x:c r="C44" s="1"/>
+      <x:c r="D44" s="1"/>
+      <x:c r="E44" s="1"/>
+      <x:c r="F44" s="1"/>
+      <x:c r="G44" s="1"/>
+      <x:c r="H44" s="1"/>
+      <x:c r="I44" s="1"/>
+      <x:c r="J44" s="1"/>
+      <x:c r="K44" s="1"/>
+      <x:c r="L44" s="1"/>
+    </x:row>
+    <x:row r="45" ht="22" customHeight="1">
+      <x:c r="A45" s="1"/>
+      <x:c r="B45" s="1"/>
+      <x:c r="C45" s="1"/>
+      <x:c r="D45" s="1"/>
+      <x:c r="E45" s="1"/>
+      <x:c r="F45" s="1"/>
+      <x:c r="G45" s="1"/>
+      <x:c r="H45" s="1"/>
+      <x:c r="I45" s="1"/>
+      <x:c r="J45" s="1"/>
+      <x:c r="K45" s="1"/>
+      <x:c r="L45" s="1"/>
+    </x:row>
+    <x:row r="46" ht="22" customHeight="1">
+      <x:c r="A46" s="1"/>
+      <x:c r="B46" s="1"/>
+      <x:c r="C46" s="1"/>
+      <x:c r="D46" s="1"/>
+      <x:c r="E46" s="1"/>
+      <x:c r="F46" s="1"/>
+      <x:c r="G46" s="1"/>
+      <x:c r="H46" s="1"/>
+      <x:c r="I46" s="1"/>
+      <x:c r="J46" s="1"/>
+      <x:c r="K46" s="1"/>
+      <x:c r="L46" s="1"/>
+    </x:row>
+    <x:row r="47" ht="22" customHeight="1">
+      <x:c r="A47" s="1"/>
+      <x:c r="B47" s="1"/>
+      <x:c r="C47" s="1"/>
+      <x:c r="D47" s="1"/>
+      <x:c r="E47" s="1"/>
+      <x:c r="F47" s="1"/>
+      <x:c r="G47" s="1"/>
+      <x:c r="H47" s="1"/>
+      <x:c r="I47" s="1"/>
+      <x:c r="J47" s="1"/>
+      <x:c r="K47" s="1"/>
+      <x:c r="L47" s="1"/>
+    </x:row>
+    <x:row r="48" ht="22" customHeight="1">
+      <x:c r="A48" s="1"/>
+      <x:c r="B48" s="1"/>
+      <x:c r="C48" s="1"/>
+      <x:c r="D48" s="1"/>
+      <x:c r="E48" s="1"/>
+      <x:c r="F48" s="1"/>
+      <x:c r="G48" s="1"/>
+      <x:c r="H48" s="1"/>
+      <x:c r="I48" s="1"/>
+      <x:c r="J48" s="1"/>
+      <x:c r="K48" s="1"/>
+      <x:c r="L48" s="1"/>
+    </x:row>
+    <x:row r="49" ht="22" customHeight="1">
+      <x:c r="A49" s="1"/>
+      <x:c r="B49" s="1"/>
+      <x:c r="C49" s="1"/>
+      <x:c r="D49" s="1"/>
+      <x:c r="E49" s="1"/>
+      <x:c r="F49" s="1"/>
+      <x:c r="G49" s="1"/>
+      <x:c r="H49" s="1"/>
+      <x:c r="I49" s="1"/>
+      <x:c r="J49" s="1"/>
+      <x:c r="K49" s="1"/>
+      <x:c r="L49" s="1"/>
+    </x:row>
+    <x:row r="50" ht="22" customHeight="1">
+      <x:c r="A50" s="1"/>
+      <x:c r="B50" s="1"/>
+      <x:c r="C50" s="1"/>
+      <x:c r="D50" s="1"/>
+      <x:c r="E50" s="1"/>
+      <x:c r="F50" s="1"/>
+      <x:c r="G50" s="1"/>
+      <x:c r="H50" s="1"/>
+      <x:c r="I50" s="1"/>
+      <x:c r="J50" s="1"/>
+      <x:c r="K50" s="1"/>
+      <x:c r="L50" s="1"/>
+    </x:row>
+    <x:row r="51" ht="22" customHeight="1">
+      <x:c r="A51" s="1"/>
+      <x:c r="B51" s="1"/>
+      <x:c r="C51" s="1"/>
+      <x:c r="D51" s="1"/>
+      <x:c r="E51" s="1"/>
+      <x:c r="F51" s="1"/>
+      <x:c r="G51" s="1"/>
+      <x:c r="H51" s="1"/>
+      <x:c r="I51" s="1"/>
+      <x:c r="J51" s="1"/>
+      <x:c r="K51" s="1"/>
+      <x:c r="L51" s="1"/>
+    </x:row>
+    <x:row r="52" ht="22" customHeight="1">
+      <x:c r="A52" s="1"/>
+      <x:c r="B52" s="1"/>
+      <x:c r="C52" s="1"/>
+      <x:c r="D52" s="1"/>
+      <x:c r="E52" s="1"/>
+      <x:c r="F52" s="1"/>
+      <x:c r="G52" s="1"/>
+      <x:c r="H52" s="1"/>
+      <x:c r="I52" s="1"/>
+      <x:c r="J52" s="1"/>
+      <x:c r="K52" s="1"/>
+      <x:c r="L52" s="1"/>
+    </x:row>
+    <x:row r="53" ht="22" customHeight="1">
+      <x:c r="A53" s="1"/>
+      <x:c r="B53" s="1"/>
+      <x:c r="C53" s="1"/>
+      <x:c r="D53" s="1"/>
+      <x:c r="E53" s="1"/>
+      <x:c r="F53" s="1"/>
+      <x:c r="G53" s="1"/>
+      <x:c r="H53" s="1"/>
+      <x:c r="I53" s="1"/>
+      <x:c r="J53" s="1"/>
+      <x:c r="K53" s="1"/>
+      <x:c r="L53" s="1"/>
+    </x:row>
+    <x:row r="54" ht="22" customHeight="1">
+      <x:c r="A54" s="1"/>
+      <x:c r="B54" s="1"/>
+      <x:c r="C54" s="1"/>
+      <x:c r="D54" s="1"/>
+      <x:c r="E54" s="1"/>
+      <x:c r="F54" s="1"/>
+      <x:c r="G54" s="1"/>
+      <x:c r="H54" s="1"/>
+      <x:c r="I54" s="1"/>
+      <x:c r="J54" s="1"/>
+      <x:c r="K54" s="1"/>
+      <x:c r="L54" s="1"/>
+    </x:row>
+    <x:row r="55" ht="22" customHeight="1">
+      <x:c r="A55" s="1"/>
+      <x:c r="B55" s="1"/>
+      <x:c r="C55" s="1"/>
+      <x:c r="D55" s="1"/>
+      <x:c r="E55" s="1"/>
+      <x:c r="F55" s="1"/>
+      <x:c r="G55" s="1"/>
+      <x:c r="H55" s="1"/>
+      <x:c r="I55" s="1"/>
+      <x:c r="J55" s="1"/>
+      <x:c r="K55" s="1"/>
+      <x:c r="L55" s="1"/>
+    </x:row>
+    <x:row r="56" ht="22" customHeight="1">
+      <x:c r="A56" s="1"/>
+      <x:c r="B56" s="1"/>
+      <x:c r="C56" s="1"/>
+      <x:c r="D56" s="1"/>
+      <x:c r="E56" s="1"/>
+      <x:c r="F56" s="1"/>
+      <x:c r="G56" s="1"/>
+      <x:c r="H56" s="1"/>
+      <x:c r="I56" s="1"/>
+      <x:c r="J56" s="1"/>
+      <x:c r="K56" s="1"/>
+      <x:c r="L56" s="1"/>
+    </x:row>
+    <x:row r="57" ht="22" customHeight="1">
+      <x:c r="A57" s="1"/>
+      <x:c r="B57" s="1"/>
+      <x:c r="C57" s="1"/>
+      <x:c r="D57" s="1"/>
+      <x:c r="E57" s="1"/>
+      <x:c r="F57" s="1"/>
+      <x:c r="G57" s="1"/>
+      <x:c r="H57" s="1"/>
+      <x:c r="I57" s="1"/>
+      <x:c r="J57" s="1"/>
+      <x:c r="K57" s="1"/>
+      <x:c r="L57" s="1"/>
+    </x:row>
+    <x:row r="58" ht="22" customHeight="1">
+      <x:c r="A58" s="1"/>
+      <x:c r="B58" s="1"/>
+      <x:c r="C58" s="1"/>
+      <x:c r="D58" s="1"/>
+      <x:c r="E58" s="1"/>
+      <x:c r="F58" s="1"/>
+      <x:c r="G58" s="1"/>
+      <x:c r="H58" s="1"/>
+      <x:c r="I58" s="1"/>
+      <x:c r="J58" s="1"/>
+      <x:c r="K58" s="1"/>
+      <x:c r="L58" s="1"/>
+    </x:row>
+    <x:row r="59" ht="22" customHeight="1">
+      <x:c r="A59" s="1"/>
+      <x:c r="B59" s="1"/>
+      <x:c r="C59" s="1"/>
+      <x:c r="D59" s="1"/>
+      <x:c r="E59" s="1"/>
+      <x:c r="F59" s="1"/>
+      <x:c r="G59" s="1"/>
+      <x:c r="H59" s="1"/>
+      <x:c r="I59" s="1"/>
+      <x:c r="J59" s="1"/>
+      <x:c r="K59" s="1"/>
+      <x:c r="L59" s="1"/>
+    </x:row>
+    <x:row r="60" ht="22" customHeight="1">
+      <x:c r="A60" s="1"/>
+      <x:c r="B60" s="1"/>
+      <x:c r="C60" s="1"/>
+      <x:c r="D60" s="1"/>
+      <x:c r="E60" s="1"/>
+      <x:c r="F60" s="1"/>
+      <x:c r="G60" s="1"/>
+      <x:c r="H60" s="1"/>
+      <x:c r="I60" s="1"/>
+      <x:c r="J60" s="1"/>
+      <x:c r="K60" s="1"/>
+      <x:c r="L60" s="1"/>
+    </x:row>
+    <x:row r="61" ht="22" customHeight="1">
+      <x:c r="A61" s="1"/>
+      <x:c r="B61" s="1"/>
+      <x:c r="C61" s="1"/>
+      <x:c r="D61" s="1"/>
+      <x:c r="E61" s="1"/>
+      <x:c r="F61" s="1"/>
+      <x:c r="G61" s="1"/>
+      <x:c r="H61" s="1"/>
+      <x:c r="I61" s="1"/>
+      <x:c r="J61" s="1"/>
+      <x:c r="K61" s="1"/>
+      <x:c r="L61" s="1"/>
+    </x:row>
+    <x:row r="62" ht="22" customHeight="1">
+      <x:c r="A62" s="1"/>
+      <x:c r="B62" s="1"/>
+      <x:c r="C62" s="1"/>
+      <x:c r="D62" s="1"/>
+      <x:c r="E62" s="1"/>
+      <x:c r="F62" s="1"/>
+      <x:c r="G62" s="1"/>
+      <x:c r="H62" s="1"/>
+      <x:c r="I62" s="1"/>
+      <x:c r="J62" s="1"/>
+      <x:c r="K62" s="1"/>
+      <x:c r="L62" s="1"/>
+    </x:row>
+    <x:row r="63" ht="22" customHeight="1">
+      <x:c r="A63" s="1"/>
+      <x:c r="B63" s="1"/>
+      <x:c r="C63" s="1"/>
+      <x:c r="D63" s="1"/>
+      <x:c r="E63" s="1"/>
+      <x:c r="F63" s="1"/>
+      <x:c r="G63" s="1"/>
+      <x:c r="H63" s="1"/>
+      <x:c r="I63" s="1"/>
+      <x:c r="J63" s="1"/>
+      <x:c r="K63" s="1"/>
+      <x:c r="L63" s="1"/>
+    </x:row>
+    <x:row r="64" ht="22" customHeight="1">
+      <x:c r="A64" s="1"/>
+      <x:c r="B64" s="1"/>
+      <x:c r="C64" s="1"/>
+      <x:c r="D64" s="1"/>
+      <x:c r="E64" s="1"/>
+      <x:c r="F64" s="1"/>
+      <x:c r="G64" s="1"/>
+      <x:c r="H64" s="1"/>
+      <x:c r="I64" s="1"/>
+      <x:c r="J64" s="1"/>
+      <x:c r="K64" s="1"/>
+      <x:c r="L64" s="1"/>
+    </x:row>
+    <x:row r="65" ht="22" customHeight="1">
+      <x:c r="A65" s="1"/>
+      <x:c r="B65" s="1"/>
+      <x:c r="C65" s="1"/>
+      <x:c r="D65" s="1"/>
+      <x:c r="E65" s="1"/>
+      <x:c r="F65" s="1"/>
+      <x:c r="G65" s="1"/>
+      <x:c r="H65" s="1"/>
+      <x:c r="I65" s="1"/>
+      <x:c r="J65" s="1"/>
+      <x:c r="K65" s="1"/>
+      <x:c r="L65" s="1"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="D4:F4"/>
+    <x:mergeCell ref="C24:K26"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="3" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="3" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="27" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="27" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="27" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="27" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="27" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="27" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="27" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="17" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="17" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="17" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="22" customHeight="1">
+      <x:c r="A1" s="1"/>
+      <x:c r="B1" s="1"/>
+      <x:c r="C1" s="1"/>
+      <x:c r="D1" s="1"/>
+      <x:c r="E1" s="1"/>
+      <x:c r="F1" s="1"/>
+      <x:c r="G1" s="1"/>
+      <x:c r="H1" s="1"/>
+      <x:c r="I1" s="1"/>
+      <x:c r="J1" s="1"/>
+      <x:c r="K1" s="1"/>
+      <x:c r="L1" s="1"/>
+    </x:row>
+    <x:row r="2" ht="22" customHeight="1">
+      <x:c r="A2" s="1"/>
+      <x:c r="B2" s="1"/>
+      <x:c r="C2" s="2" t="str">
+        <x:v>Decision ownership and approval</x:v>
+      </x:c>
+      <x:c r="D2" s="1"/>
+      <x:c r="E2" s="1"/>
+      <x:c r="F2" s="1"/>
+      <x:c r="G2" s="1"/>
+      <x:c r="H2" s="1"/>
+      <x:c r="I2" s="1"/>
+      <x:c r="J2" s="1"/>
+      <x:c r="K2" s="1"/>
+      <x:c r="L2" s="1"/>
+    </x:row>
+    <x:row r="3" ht="22" customHeight="1">
+      <x:c r="A3" s="1"/>
+      <x:c r="B3" s="1"/>
+      <x:c r="C3" s="3"/>
+      <x:c r="D3" s="3"/>
+      <x:c r="E3" s="3"/>
+      <x:c r="F3" s="3"/>
+      <x:c r="G3" s="3"/>
+      <x:c r="H3" s="3"/>
+      <x:c r="I3" s="3"/>
+      <x:c r="J3" s="3"/>
+      <x:c r="K3" s="3"/>
+      <x:c r="L3" s="3"/>
+    </x:row>
+    <x:row r="4" ht="22" customHeight="1">
+      <x:c r="A4" s="1"/>
+      <x:c r="B4" s="1"/>
+      <x:c r="C4" s="1" t="str">
+        <x:v>Roles and deadlines are proposed within a synthetic case.</x:v>
+      </x:c>
+      <x:c r="D4" s="1"/>
+      <x:c r="E4" s="1"/>
+      <x:c r="F4" s="1"/>
+      <x:c r="G4" s="1"/>
+      <x:c r="H4" s="1"/>
+      <x:c r="I4" s="1"/>
+      <x:c r="J4" s="1"/>
+      <x:c r="K4" s="1"/>
+      <x:c r="L4" s="1"/>
+    </x:row>
+    <x:row r="5" ht="22" customHeight="1">
+      <x:c r="A5" s="1"/>
+      <x:c r="B5" s="1"/>
+      <x:c r="C5" s="1"/>
+      <x:c r="D5" s="1"/>
+      <x:c r="E5" s="1"/>
+      <x:c r="F5" s="1"/>
+      <x:c r="G5" s="1"/>
+      <x:c r="H5" s="1"/>
+      <x:c r="I5" s="1"/>
+      <x:c r="J5" s="1"/>
+      <x:c r="K5" s="1"/>
+      <x:c r="L5" s="1"/>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="1"/>
+      <x:c r="B6" s="1"/>
+      <x:c r="C6" s="23" t="str">
+        <x:v>Action</x:v>
+      </x:c>
+      <x:c r="D6" s="23" t="str">
+        <x:v>Proposed owner</x:v>
+      </x:c>
+      <x:c r="E6" s="23" t="str">
+        <x:v>Due from approval</x:v>
+      </x:c>
+      <x:c r="F6" s="23" t="str">
+        <x:v>Trigger / evidence</x:v>
+      </x:c>
+      <x:c r="G6" s="23" t="str">
+        <x:v>Approval needed</x:v>
+      </x:c>
+      <x:c r="H6" s="23" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="I6" s="23" t="str">
+        <x:v>Evidence link</x:v>
+      </x:c>
+      <x:c r="J6" s="1"/>
+      <x:c r="K6" s="1"/>
+      <x:c r="L6" s="1"/>
+    </x:row>
+    <x:row r="7" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A7" s="1"/>
+      <x:c r="B7" s="1"/>
+      <x:c r="C7" s="5" t="str">
+        <x:v>Obtain purchase and lease quotes</x:v>
+      </x:c>
+      <x:c r="D7" s="5" t="str">
+        <x:v>Fleet + Procurement</x:v>
+      </x:c>
+      <x:c r="E7" s="5" t="str">
+        <x:v>Day 10</x:v>
+      </x:c>
+      <x:c r="F7" s="5" t="str">
+        <x:v>Comparable service and coverage</x:v>
+      </x:c>
+      <x:c r="G7" s="5" t="str">
+        <x:v>Procurement lead</x:v>
+      </x:c>
+      <x:c r="H7" s="5" t="str">
+        <x:v>Proposed</x:v>
+      </x:c>
+      <x:c r="I7" s="5" t="str"/>
+      <x:c r="J7" s="1"/>
+      <x:c r="K7" s="1"/>
+      <x:c r="L7" s="1"/>
+    </x:row>
+    <x:row r="8" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A8" s="1"/>
+      <x:c r="B8" s="1"/>
+      <x:c r="C8" s="5" t="str">
+        <x:v>Approve capital and liquidity</x:v>
+      </x:c>
+      <x:c r="D8" s="5" t="str">
+        <x:v>Finance + Treasury</x:v>
+      </x:c>
+      <x:c r="E8" s="5" t="str">
+        <x:v>Day 15</x:v>
+      </x:c>
+      <x:c r="F8" s="5" t="str">
+        <x:v>Net upfront cash within $700k</x:v>
+      </x:c>
+      <x:c r="G8" s="5" t="str">
+        <x:v>Investment committee</x:v>
+      </x:c>
+      <x:c r="H8" s="5" t="str">
+        <x:v>Proposed</x:v>
+      </x:c>
+      <x:c r="I8" s="5" t="str"/>
+      <x:c r="J8" s="1"/>
+      <x:c r="K8" s="1"/>
+      <x:c r="L8" s="1"/>
+    </x:row>
+    <x:row r="9" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A9" s="1"/>
+      <x:c r="B9" s="1"/>
+      <x:c r="C9" s="5" t="str">
+        <x:v>Verify tax and residual assumptions</x:v>
+      </x:c>
+      <x:c r="D9" s="5" t="str">
+        <x:v>Finance</x:v>
+      </x:c>
+      <x:c r="E9" s="5" t="str">
+        <x:v>Before commitment</x:v>
+      </x:c>
+      <x:c r="F9" s="5" t="str">
+        <x:v>Tax-adjusted economics reviewed</x:v>
+      </x:c>
+      <x:c r="G9" s="5" t="str">
+        <x:v>Finance lead</x:v>
+      </x:c>
+      <x:c r="H9" s="5" t="str">
+        <x:v>Proposed</x:v>
+      </x:c>
+      <x:c r="I9" s="5" t="str"/>
+      <x:c r="J9" s="1"/>
+      <x:c r="K9" s="1"/>
+      <x:c r="L9" s="1"/>
+    </x:row>
+    <x:row r="10" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A10" s="1"/>
+      <x:c r="B10" s="1"/>
+      <x:c r="C10" s="5" t="str">
+        <x:v>Review benefits after commissioning</x:v>
+      </x:c>
+      <x:c r="D10" s="5" t="str">
+        <x:v>Fleet + Finance</x:v>
+      </x:c>
+      <x:c r="E10" s="5" t="str">
+        <x:v>Days 30 / 90 / 180</x:v>
+      </x:c>
+      <x:c r="F10" s="5" t="str">
+        <x:v>Maintenance, mpg, downtime vs plan</x:v>
+      </x:c>
+      <x:c r="G10" s="5" t="str">
+        <x:v>Operations lead</x:v>
+      </x:c>
+      <x:c r="H10" s="5" t="str">
+        <x:v>Proposed</x:v>
+      </x:c>
+      <x:c r="I10" s="5" t="str"/>
+      <x:c r="J10" s="1"/>
+      <x:c r="K10" s="1"/>
+      <x:c r="L10" s="1"/>
+    </x:row>
+    <x:row r="11" ht="22" customHeight="1">
+      <x:c r="A11" s="1"/>
+      <x:c r="B11" s="1"/>
+      <x:c r="C11" s="1"/>
+      <x:c r="D11" s="1"/>
+      <x:c r="E11" s="1"/>
+      <x:c r="F11" s="1"/>
+      <x:c r="G11" s="1"/>
+      <x:c r="H11" s="1"/>
+      <x:c r="I11" s="1"/>
+      <x:c r="J11" s="1"/>
+      <x:c r="K11" s="1"/>
+      <x:c r="L11" s="1"/>
+    </x:row>
+    <x:row r="12" ht="22" customHeight="1">
+      <x:c r="A12" s="1"/>
+      <x:c r="B12" s="1"/>
+      <x:c r="C12" s="1"/>
+      <x:c r="D12" s="1"/>
+      <x:c r="E12" s="1"/>
+      <x:c r="F12" s="1"/>
+      <x:c r="G12" s="1"/>
+      <x:c r="H12" s="1"/>
+      <x:c r="I12" s="1"/>
+      <x:c r="J12" s="1"/>
+      <x:c r="K12" s="1"/>
+      <x:c r="L12" s="1"/>
+    </x:row>
+    <x:row r="13" ht="22" customHeight="1">
+      <x:c r="A13" s="1"/>
+      <x:c r="B13" s="1"/>
+      <x:c r="C13" s="1"/>
+      <x:c r="D13" s="1"/>
+      <x:c r="E13" s="1"/>
+      <x:c r="F13" s="1"/>
+      <x:c r="G13" s="1"/>
+      <x:c r="H13" s="1"/>
+      <x:c r="I13" s="1"/>
+      <x:c r="J13" s="1"/>
+      <x:c r="K13" s="1"/>
+      <x:c r="L13" s="1"/>
+    </x:row>
+    <x:row r="14" ht="22" customHeight="1">
+      <x:c r="A14" s="1"/>
+      <x:c r="B14" s="1"/>
+      <x:c r="C14" s="1"/>
+      <x:c r="D14" s="1"/>
+      <x:c r="E14" s="1"/>
+      <x:c r="F14" s="1"/>
+      <x:c r="G14" s="1"/>
+      <x:c r="H14" s="1"/>
+      <x:c r="I14" s="1"/>
+      <x:c r="J14" s="1"/>
+      <x:c r="K14" s="1"/>
+      <x:c r="L14" s="1"/>
+    </x:row>
+    <x:row r="15" ht="22" customHeight="1">
+      <x:c r="A15" s="1"/>
+      <x:c r="B15" s="1"/>
+      <x:c r="C15" s="1"/>
+      <x:c r="D15" s="1"/>
+      <x:c r="E15" s="1"/>
+      <x:c r="F15" s="1"/>
+      <x:c r="G15" s="1"/>
+      <x:c r="H15" s="1"/>
+      <x:c r="I15" s="1"/>
+      <x:c r="J15" s="1"/>
+      <x:c r="K15" s="1"/>
+      <x:c r="L15" s="1"/>
+    </x:row>
+    <x:row r="16" ht="22" customHeight="1">
+      <x:c r="A16" s="1"/>
+      <x:c r="B16" s="1"/>
+      <x:c r="C16" s="1"/>
+      <x:c r="D16" s="1"/>
+      <x:c r="E16" s="1"/>
+      <x:c r="F16" s="1"/>
+      <x:c r="G16" s="1"/>
+      <x:c r="H16" s="1"/>
+      <x:c r="I16" s="1"/>
+      <x:c r="J16" s="1"/>
+      <x:c r="K16" s="1"/>
+      <x:c r="L16" s="1"/>
+    </x:row>
+    <x:row r="17" ht="22" customHeight="1">
+      <x:c r="A17" s="1"/>
+      <x:c r="B17" s="1"/>
+      <x:c r="C17" s="1"/>
+      <x:c r="D17" s="1"/>
+      <x:c r="E17" s="1"/>
+      <x:c r="F17" s="1"/>
+      <x:c r="G17" s="1"/>
+      <x:c r="H17" s="1"/>
+      <x:c r="I17" s="1"/>
+      <x:c r="J17" s="1"/>
+      <x:c r="K17" s="1"/>
+      <x:c r="L17" s="1"/>
+    </x:row>
+    <x:row r="18" ht="22" customHeight="1">
+      <x:c r="A18" s="1"/>
+      <x:c r="B18" s="1"/>
+      <x:c r="C18" s="1"/>
+      <x:c r="D18" s="1"/>
+      <x:c r="E18" s="1"/>
+      <x:c r="F18" s="1"/>
+      <x:c r="G18" s="1"/>
+      <x:c r="H18" s="1"/>
+      <x:c r="I18" s="1"/>
+      <x:c r="J18" s="1"/>
+      <x:c r="K18" s="1"/>
+      <x:c r="L18" s="1"/>
+    </x:row>
+    <x:row r="19" ht="22" customHeight="1">
+      <x:c r="A19" s="1"/>
+      <x:c r="B19" s="1"/>
+      <x:c r="C19" s="1"/>
+      <x:c r="D19" s="1"/>
+      <x:c r="E19" s="1"/>
+      <x:c r="F19" s="1"/>
+      <x:c r="G19" s="1"/>
+      <x:c r="H19" s="1"/>
+      <x:c r="I19" s="1"/>
+      <x:c r="J19" s="1"/>
+      <x:c r="K19" s="1"/>
+      <x:c r="L19" s="1"/>
+    </x:row>
+    <x:row r="20" ht="22" customHeight="1">
+      <x:c r="A20" s="1"/>
+      <x:c r="B20" s="1"/>
+      <x:c r="C20" s="1"/>
+      <x:c r="D20" s="1"/>
+      <x:c r="E20" s="1"/>
+      <x:c r="F20" s="1"/>
+      <x:c r="G20" s="1"/>
+      <x:c r="H20" s="1"/>
+      <x:c r="I20" s="1"/>
+      <x:c r="J20" s="1"/>
+      <x:c r="K20" s="1"/>
+      <x:c r="L20" s="1"/>
+    </x:row>
+    <x:row r="21" ht="22" customHeight="1">
+      <x:c r="A21" s="1"/>
+      <x:c r="B21" s="1"/>
+      <x:c r="C21" s="1"/>
+      <x:c r="D21" s="1"/>
+      <x:c r="E21" s="1"/>
+      <x:c r="F21" s="1"/>
+      <x:c r="G21" s="1"/>
+      <x:c r="H21" s="1"/>
+      <x:c r="I21" s="1"/>
+      <x:c r="J21" s="1"/>
+      <x:c r="K21" s="1"/>
+      <x:c r="L21" s="1"/>
+    </x:row>
+    <x:row r="22" ht="22" customHeight="1">
+      <x:c r="A22" s="1"/>
+      <x:c r="B22" s="1"/>
+      <x:c r="C22" s="1"/>
+      <x:c r="D22" s="1"/>
+      <x:c r="E22" s="1"/>
+      <x:c r="F22" s="1"/>
+      <x:c r="G22" s="1"/>
+      <x:c r="H22" s="1"/>
+      <x:c r="I22" s="1"/>
+      <x:c r="J22" s="1"/>
+      <x:c r="K22" s="1"/>
+      <x:c r="L22" s="1"/>
+    </x:row>
+    <x:row r="23" ht="22" customHeight="1">
+      <x:c r="A23" s="1"/>
+      <x:c r="B23" s="1"/>
+      <x:c r="C23" s="1"/>
+      <x:c r="D23" s="1"/>
+      <x:c r="E23" s="1"/>
+      <x:c r="F23" s="1"/>
+      <x:c r="G23" s="1"/>
+      <x:c r="H23" s="1"/>
+      <x:c r="I23" s="1"/>
+      <x:c r="J23" s="1"/>
+      <x:c r="K23" s="1"/>
+      <x:c r="L23" s="1"/>
+    </x:row>
+    <x:row r="24" ht="22" customHeight="1">
+      <x:c r="A24" s="1"/>
+      <x:c r="B24" s="1"/>
+      <x:c r="C24" s="1"/>
+      <x:c r="D24" s="1"/>
+      <x:c r="E24" s="1"/>
+      <x:c r="F24" s="1"/>
+      <x:c r="G24" s="1"/>
+      <x:c r="H24" s="1"/>
+      <x:c r="I24" s="1"/>
+      <x:c r="J24" s="1"/>
+      <x:c r="K24" s="1"/>
+      <x:c r="L24" s="1"/>
+    </x:row>
+    <x:row r="25" ht="22" customHeight="1">
+      <x:c r="A25" s="1"/>
+      <x:c r="B25" s="1"/>
+      <x:c r="C25" s="1"/>
+      <x:c r="D25" s="1"/>
+      <x:c r="E25" s="1"/>
+      <x:c r="F25" s="1"/>
+      <x:c r="G25" s="1"/>
+      <x:c r="H25" s="1"/>
+      <x:c r="I25" s="1"/>
+      <x:c r="J25" s="1"/>
+      <x:c r="K25" s="1"/>
+      <x:c r="L25" s="1"/>
+    </x:row>
+    <x:row r="26" ht="22" customHeight="1">
+      <x:c r="A26" s="1"/>
+      <x:c r="B26" s="1"/>
+      <x:c r="C26" s="1"/>
+      <x:c r="D26" s="1"/>
+      <x:c r="E26" s="1"/>
+      <x:c r="F26" s="1"/>
+      <x:c r="G26" s="1"/>
+      <x:c r="H26" s="1"/>
+      <x:c r="I26" s="1"/>
+      <x:c r="J26" s="1"/>
+      <x:c r="K26" s="1"/>
+      <x:c r="L26" s="1"/>
+    </x:row>
+    <x:row r="27" ht="22" customHeight="1">
+      <x:c r="A27" s="1"/>
+      <x:c r="B27" s="1"/>
+      <x:c r="C27" s="1"/>
+      <x:c r="D27" s="1"/>
+      <x:c r="E27" s="1"/>
+      <x:c r="F27" s="1"/>
+      <x:c r="G27" s="1"/>
+      <x:c r="H27" s="1"/>
+      <x:c r="I27" s="1"/>
+      <x:c r="J27" s="1"/>
+      <x:c r="K27" s="1"/>
+      <x:c r="L27" s="1"/>
+    </x:row>
+    <x:row r="28" ht="22" customHeight="1">
+      <x:c r="A28" s="1"/>
+      <x:c r="B28" s="1"/>
+      <x:c r="C28" s="1"/>
+      <x:c r="D28" s="1"/>
+      <x:c r="E28" s="1"/>
+      <x:c r="F28" s="1"/>
+      <x:c r="G28" s="1"/>
+      <x:c r="H28" s="1"/>
+      <x:c r="I28" s="1"/>
+      <x:c r="J28" s="1"/>
+      <x:c r="K28" s="1"/>
+      <x:c r="L28" s="1"/>
+    </x:row>
+    <x:row r="29" ht="22" customHeight="1">
+      <x:c r="A29" s="1"/>
+      <x:c r="B29" s="1"/>
+      <x:c r="C29" s="1"/>
+      <x:c r="D29" s="1"/>
+      <x:c r="E29" s="1"/>
+      <x:c r="F29" s="1"/>
+      <x:c r="G29" s="1"/>
+      <x:c r="H29" s="1"/>
+      <x:c r="I29" s="1"/>
+      <x:c r="J29" s="1"/>
+      <x:c r="K29" s="1"/>
+      <x:c r="L29" s="1"/>
+    </x:row>
+    <x:row r="30" ht="22" customHeight="1">
+      <x:c r="A30" s="1"/>
+      <x:c r="B30" s="1"/>
+      <x:c r="C30" s="1"/>
+      <x:c r="D30" s="1"/>
+      <x:c r="E30" s="1"/>
+      <x:c r="F30" s="1"/>
+      <x:c r="G30" s="1"/>
+      <x:c r="H30" s="1"/>
+      <x:c r="I30" s="1"/>
+      <x:c r="J30" s="1"/>
+      <x:c r="K30" s="1"/>
+      <x:c r="L30" s="1"/>
+    </x:row>
+    <x:row r="31" ht="22" customHeight="1">
+      <x:c r="A31" s="1"/>
+      <x:c r="B31" s="1"/>
+      <x:c r="C31" s="1"/>
+      <x:c r="D31" s="1"/>
+      <x:c r="E31" s="1"/>
+      <x:c r="F31" s="1"/>
+      <x:c r="G31" s="1"/>
+      <x:c r="H31" s="1"/>
+      <x:c r="I31" s="1"/>
+      <x:c r="J31" s="1"/>
+      <x:c r="K31" s="1"/>
+      <x:c r="L31" s="1"/>
+    </x:row>
+    <x:row r="32" ht="22" customHeight="1">
+      <x:c r="A32" s="1"/>
+      <x:c r="B32" s="1"/>
+      <x:c r="C32" s="1"/>
+      <x:c r="D32" s="1"/>
+      <x:c r="E32" s="1"/>
+      <x:c r="F32" s="1"/>
+      <x:c r="G32" s="1"/>
+      <x:c r="H32" s="1"/>
+      <x:c r="I32" s="1"/>
+      <x:c r="J32" s="1"/>
+      <x:c r="K32" s="1"/>
+      <x:c r="L32" s="1"/>
+    </x:row>
+    <x:row r="33" ht="22" customHeight="1">
+      <x:c r="A33" s="1"/>
+      <x:c r="B33" s="1"/>
+      <x:c r="C33" s="1"/>
+      <x:c r="D33" s="1"/>
+      <x:c r="E33" s="1"/>
+      <x:c r="F33" s="1"/>
+      <x:c r="G33" s="1"/>
+      <x:c r="H33" s="1"/>
+      <x:c r="I33" s="1"/>
+      <x:c r="J33" s="1"/>
+      <x:c r="K33" s="1"/>
+      <x:c r="L33" s="1"/>
+    </x:row>
+    <x:row r="34" ht="22" customHeight="1">
+      <x:c r="A34" s="1"/>
+      <x:c r="B34" s="1"/>
+      <x:c r="C34" s="1"/>
+      <x:c r="D34" s="1"/>
+      <x:c r="E34" s="1"/>
+      <x:c r="F34" s="1"/>
+      <x:c r="G34" s="1"/>
+      <x:c r="H34" s="1"/>
+      <x:c r="I34" s="1"/>
+      <x:c r="J34" s="1"/>
+      <x:c r="K34" s="1"/>
+      <x:c r="L34" s="1"/>
+    </x:row>
+    <x:row r="35" ht="22" customHeight="1">
+      <x:c r="A35" s="1"/>
+      <x:c r="B35" s="1"/>
+      <x:c r="C35" s="1"/>
+      <x:c r="D35" s="1"/>
+      <x:c r="E35" s="1"/>
+      <x:c r="F35" s="1"/>
+      <x:c r="G35" s="1"/>
+      <x:c r="H35" s="1"/>
+      <x:c r="I35" s="1"/>
+      <x:c r="J35" s="1"/>
+      <x:c r="K35" s="1"/>
+      <x:c r="L35" s="1"/>
+    </x:row>
+    <x:row r="36" ht="22" customHeight="1">
+      <x:c r="A36" s="1"/>
+      <x:c r="B36" s="1"/>
+      <x:c r="C36" s="1"/>
+      <x:c r="D36" s="1"/>
+      <x:c r="E36" s="1"/>
+      <x:c r="F36" s="1"/>
+      <x:c r="G36" s="1"/>
+      <x:c r="H36" s="1"/>
+      <x:c r="I36" s="1"/>
+      <x:c r="J36" s="1"/>
+      <x:c r="K36" s="1"/>
+      <x:c r="L36" s="1"/>
+    </x:row>
+    <x:row r="37" ht="22" customHeight="1">
+      <x:c r="A37" s="1"/>
+      <x:c r="B37" s="1"/>
+      <x:c r="C37" s="1"/>
+      <x:c r="D37" s="1"/>
+      <x:c r="E37" s="1"/>
+      <x:c r="F37" s="1"/>
+      <x:c r="G37" s="1"/>
+      <x:c r="H37" s="1"/>
+      <x:c r="I37" s="1"/>
+      <x:c r="J37" s="1"/>
+      <x:c r="K37" s="1"/>
+      <x:c r="L37" s="1"/>
+    </x:row>
+    <x:row r="38" ht="22" customHeight="1">
+      <x:c r="A38" s="1"/>
+      <x:c r="B38" s="1"/>
+      <x:c r="C38" s="1"/>
+      <x:c r="D38" s="1"/>
+      <x:c r="E38" s="1"/>
+      <x:c r="F38" s="1"/>
+      <x:c r="G38" s="1"/>
+      <x:c r="H38" s="1"/>
+      <x:c r="I38" s="1"/>
+      <x:c r="J38" s="1"/>
+      <x:c r="K38" s="1"/>
+      <x:c r="L38" s="1"/>
+    </x:row>
+    <x:row r="39" ht="22" customHeight="1">
+      <x:c r="A39" s="1"/>
+      <x:c r="B39" s="1"/>
+      <x:c r="C39" s="1"/>
+      <x:c r="D39" s="1"/>
+      <x:c r="E39" s="1"/>
+      <x:c r="F39" s="1"/>
+      <x:c r="G39" s="1"/>
+      <x:c r="H39" s="1"/>
+      <x:c r="I39" s="1"/>
+      <x:c r="J39" s="1"/>
+      <x:c r="K39" s="1"/>
+      <x:c r="L39" s="1"/>
+    </x:row>
+    <x:row r="40" ht="22" customHeight="1">
+      <x:c r="A40" s="1"/>
+      <x:c r="B40" s="1"/>
+      <x:c r="C40" s="1"/>
+      <x:c r="D40" s="1"/>
+      <x:c r="E40" s="1"/>
+      <x:c r="F40" s="1"/>
+      <x:c r="G40" s="1"/>
+      <x:c r="H40" s="1"/>
+      <x:c r="I40" s="1"/>
+      <x:c r="J40" s="1"/>
+      <x:c r="K40" s="1"/>
+      <x:c r="L40" s="1"/>
+    </x:row>
+    <x:row r="41" ht="22" customHeight="1">
+      <x:c r="A41" s="1"/>
+      <x:c r="B41" s="1"/>
+      <x:c r="C41" s="1"/>
+      <x:c r="D41" s="1"/>
+      <x:c r="E41" s="1"/>
+      <x:c r="F41" s="1"/>
+      <x:c r="G41" s="1"/>
+      <x:c r="H41" s="1"/>
+      <x:c r="I41" s="1"/>
+      <x:c r="J41" s="1"/>
+      <x:c r="K41" s="1"/>
+      <x:c r="L41" s="1"/>
+    </x:row>
+    <x:row r="42" ht="22" customHeight="1">
+      <x:c r="A42" s="1"/>
+      <x:c r="B42" s="1"/>
+      <x:c r="C42" s="1"/>
+      <x:c r="D42" s="1"/>
+      <x:c r="E42" s="1"/>
+      <x:c r="F42" s="1"/>
+      <x:c r="G42" s="1"/>
+      <x:c r="H42" s="1"/>
+      <x:c r="I42" s="1"/>
+      <x:c r="J42" s="1"/>
+      <x:c r="K42" s="1"/>
+      <x:c r="L42" s="1"/>
+    </x:row>
+    <x:row r="43" ht="22" customHeight="1">
+      <x:c r="A43" s="1"/>
+      <x:c r="B43" s="1"/>
+      <x:c r="C43" s="1"/>
+      <x:c r="D43" s="1"/>
+      <x:c r="E43" s="1"/>
+      <x:c r="F43" s="1"/>
+      <x:c r="G43" s="1"/>
+      <x:c r="H43" s="1"/>
+      <x:c r="I43" s="1"/>
+      <x:c r="J43" s="1"/>
+      <x:c r="K43" s="1"/>
+      <x:c r="L43" s="1"/>
+    </x:row>
+    <x:row r="44" ht="22" customHeight="1">
+      <x:c r="A44" s="1"/>
+      <x:c r="B44" s="1"/>
+      <x:c r="C44" s="1"/>
+      <x:c r="D44" s="1"/>
+      <x:c r="E44" s="1"/>
+      <x:c r="F44" s="1"/>
+      <x:c r="G44" s="1"/>
+      <x:c r="H44" s="1"/>
+      <x:c r="I44" s="1"/>
+      <x:c r="J44" s="1"/>
+      <x:c r="K44" s="1"/>
+      <x:c r="L44" s="1"/>
+    </x:row>
+    <x:row r="45" ht="22" customHeight="1">
+      <x:c r="A45" s="1"/>
+      <x:c r="B45" s="1"/>
+      <x:c r="C45" s="1"/>
+      <x:c r="D45" s="1"/>
+      <x:c r="E45" s="1"/>
+      <x:c r="F45" s="1"/>
+      <x:c r="G45" s="1"/>
+      <x:c r="H45" s="1"/>
+      <x:c r="I45" s="1"/>
+      <x:c r="J45" s="1"/>
+      <x:c r="K45" s="1"/>
+      <x:c r="L45" s="1"/>
+    </x:row>
+    <x:row r="46" ht="22" customHeight="1">
+      <x:c r="A46" s="1"/>
+      <x:c r="B46" s="1"/>
+      <x:c r="C46" s="1"/>
+      <x:c r="D46" s="1"/>
+      <x:c r="E46" s="1"/>
+      <x:c r="F46" s="1"/>
+      <x:c r="G46" s="1"/>
+      <x:c r="H46" s="1"/>
+      <x:c r="I46" s="1"/>
+      <x:c r="J46" s="1"/>
+      <x:c r="K46" s="1"/>
+      <x:c r="L46" s="1"/>
+    </x:row>
+    <x:row r="47" ht="22" customHeight="1">
+      <x:c r="A47" s="1"/>
+      <x:c r="B47" s="1"/>
+      <x:c r="C47" s="1"/>
+      <x:c r="D47" s="1"/>
+      <x:c r="E47" s="1"/>
+      <x:c r="F47" s="1"/>
+      <x:c r="G47" s="1"/>
+      <x:c r="H47" s="1"/>
+      <x:c r="I47" s="1"/>
+      <x:c r="J47" s="1"/>
+      <x:c r="K47" s="1"/>
+      <x:c r="L47" s="1"/>
+    </x:row>
+    <x:row r="48" ht="22" customHeight="1">
+      <x:c r="A48" s="1"/>
+      <x:c r="B48" s="1"/>
+      <x:c r="C48" s="1"/>
+      <x:c r="D48" s="1"/>
+      <x:c r="E48" s="1"/>
+      <x:c r="F48" s="1"/>
+      <x:c r="G48" s="1"/>
+      <x:c r="H48" s="1"/>
+      <x:c r="I48" s="1"/>
+      <x:c r="J48" s="1"/>
+      <x:c r="K48" s="1"/>
+      <x:c r="L48" s="1"/>
+    </x:row>
+    <x:row r="49" ht="22" customHeight="1">
+      <x:c r="A49" s="1"/>
+      <x:c r="B49" s="1"/>
+      <x:c r="C49" s="1"/>
+      <x:c r="D49" s="1"/>
+      <x:c r="E49" s="1"/>
+      <x:c r="F49" s="1"/>
+      <x:c r="G49" s="1"/>
+      <x:c r="H49" s="1"/>
+      <x:c r="I49" s="1"/>
+      <x:c r="J49" s="1"/>
+      <x:c r="K49" s="1"/>
+      <x:c r="L49" s="1"/>
+    </x:row>
+    <x:row r="50" ht="22" customHeight="1">
+      <x:c r="A50" s="1"/>
+      <x:c r="B50" s="1"/>
+      <x:c r="C50" s="1"/>
+      <x:c r="D50" s="1"/>
+      <x:c r="E50" s="1"/>
+      <x:c r="F50" s="1"/>
+      <x:c r="G50" s="1"/>
+      <x:c r="H50" s="1"/>
+      <x:c r="I50" s="1"/>
+      <x:c r="J50" s="1"/>
+      <x:c r="K50" s="1"/>
+      <x:c r="L50" s="1"/>
+    </x:row>
+    <x:row r="51" ht="22" customHeight="1">
+      <x:c r="A51" s="1"/>
+      <x:c r="B51" s="1"/>
+      <x:c r="C51" s="1"/>
+      <x:c r="D51" s="1"/>
+      <x:c r="E51" s="1"/>
+      <x:c r="F51" s="1"/>
+      <x:c r="G51" s="1"/>
+      <x:c r="H51" s="1"/>
+      <x:c r="I51" s="1"/>
+      <x:c r="J51" s="1"/>
+      <x:c r="K51" s="1"/>
+      <x:c r="L51" s="1"/>
+    </x:row>
+    <x:row r="52" ht="22" customHeight="1">
+      <x:c r="A52" s="1"/>
+      <x:c r="B52" s="1"/>
+      <x:c r="C52" s="1"/>
+      <x:c r="D52" s="1"/>
+      <x:c r="E52" s="1"/>
+      <x:c r="F52" s="1"/>
+      <x:c r="G52" s="1"/>
+      <x:c r="H52" s="1"/>
+      <x:c r="I52" s="1"/>
+      <x:c r="J52" s="1"/>
+      <x:c r="K52" s="1"/>
+      <x:c r="L52" s="1"/>
+    </x:row>
+    <x:row r="53" ht="22" customHeight="1">
+      <x:c r="A53" s="1"/>
+      <x:c r="B53" s="1"/>
+      <x:c r="C53" s="1"/>
+      <x:c r="D53" s="1"/>
+      <x:c r="E53" s="1"/>
+      <x:c r="F53" s="1"/>
+      <x:c r="G53" s="1"/>
+      <x:c r="H53" s="1"/>
+      <x:c r="I53" s="1"/>
+      <x:c r="J53" s="1"/>
+      <x:c r="K53" s="1"/>
+      <x:c r="L53" s="1"/>
+    </x:row>
+    <x:row r="54" ht="22" customHeight="1">
+      <x:c r="A54" s="1"/>
+      <x:c r="B54" s="1"/>
+      <x:c r="C54" s="1"/>
+      <x:c r="D54" s="1"/>
+      <x:c r="E54" s="1"/>
+      <x:c r="F54" s="1"/>
+      <x:c r="G54" s="1"/>
+      <x:c r="H54" s="1"/>
+      <x:c r="I54" s="1"/>
+      <x:c r="J54" s="1"/>
+      <x:c r="K54" s="1"/>
+      <x:c r="L54" s="1"/>
+    </x:row>
+    <x:row r="55" ht="22" customHeight="1">
+      <x:c r="A55" s="1"/>
+      <x:c r="B55" s="1"/>
+      <x:c r="C55" s="1"/>
+      <x:c r="D55" s="1"/>
+      <x:c r="E55" s="1"/>
+      <x:c r="F55" s="1"/>
+      <x:c r="G55" s="1"/>
+      <x:c r="H55" s="1"/>
+      <x:c r="I55" s="1"/>
+      <x:c r="J55" s="1"/>
+      <x:c r="K55" s="1"/>
+      <x:c r="L55" s="1"/>
+    </x:row>
+    <x:row r="56" ht="22" customHeight="1">
+      <x:c r="A56" s="1"/>
+      <x:c r="B56" s="1"/>
+      <x:c r="C56" s="1"/>
+      <x:c r="D56" s="1"/>
+      <x:c r="E56" s="1"/>
+      <x:c r="F56" s="1"/>
+      <x:c r="G56" s="1"/>
+      <x:c r="H56" s="1"/>
+      <x:c r="I56" s="1"/>
+      <x:c r="J56" s="1"/>
+      <x:c r="K56" s="1"/>
+      <x:c r="L56" s="1"/>
+    </x:row>
+    <x:row r="57" ht="22" customHeight="1">
+      <x:c r="A57" s="1"/>
+      <x:c r="B57" s="1"/>
+      <x:c r="C57" s="1"/>
+      <x:c r="D57" s="1"/>
+      <x:c r="E57" s="1"/>
+      <x:c r="F57" s="1"/>
+      <x:c r="G57" s="1"/>
+      <x:c r="H57" s="1"/>
+      <x:c r="I57" s="1"/>
+      <x:c r="J57" s="1"/>
+      <x:c r="K57" s="1"/>
+      <x:c r="L57" s="1"/>
+    </x:row>
+    <x:row r="58" ht="22" customHeight="1">
+      <x:c r="A58" s="1"/>
+      <x:c r="B58" s="1"/>
+      <x:c r="C58" s="1"/>
+      <x:c r="D58" s="1"/>
+      <x:c r="E58" s="1"/>
+      <x:c r="F58" s="1"/>
+      <x:c r="G58" s="1"/>
+      <x:c r="H58" s="1"/>
+      <x:c r="I58" s="1"/>
+      <x:c r="J58" s="1"/>
+      <x:c r="K58" s="1"/>
+      <x:c r="L58" s="1"/>
+    </x:row>
+    <x:row r="59" ht="22" customHeight="1">
+      <x:c r="A59" s="1"/>
+      <x:c r="B59" s="1"/>
+      <x:c r="C59" s="1"/>
+      <x:c r="D59" s="1"/>
+      <x:c r="E59" s="1"/>
+      <x:c r="F59" s="1"/>
+      <x:c r="G59" s="1"/>
+      <x:c r="H59" s="1"/>
+      <x:c r="I59" s="1"/>
+      <x:c r="J59" s="1"/>
+      <x:c r="K59" s="1"/>
+      <x:c r="L59" s="1"/>
+    </x:row>
+    <x:row r="60" ht="22" customHeight="1">
+      <x:c r="A60" s="1"/>
+      <x:c r="B60" s="1"/>
+      <x:c r="C60" s="1"/>
+      <x:c r="D60" s="1"/>
+      <x:c r="E60" s="1"/>
+      <x:c r="F60" s="1"/>
+      <x:c r="G60" s="1"/>
+      <x:c r="H60" s="1"/>
+      <x:c r="I60" s="1"/>
+      <x:c r="J60" s="1"/>
+      <x:c r="K60" s="1"/>
+      <x:c r="L60" s="1"/>
+    </x:row>
+    <x:row r="61" ht="22" customHeight="1">
+      <x:c r="A61" s="1"/>
+      <x:c r="B61" s="1"/>
+      <x:c r="C61" s="1"/>
+      <x:c r="D61" s="1"/>
+      <x:c r="E61" s="1"/>
+      <x:c r="F61" s="1"/>
+      <x:c r="G61" s="1"/>
+      <x:c r="H61" s="1"/>
+      <x:c r="I61" s="1"/>
+      <x:c r="J61" s="1"/>
+      <x:c r="K61" s="1"/>
+      <x:c r="L61" s="1"/>
+    </x:row>
+    <x:row r="62" ht="22" customHeight="1">
+      <x:c r="A62" s="1"/>
+      <x:c r="B62" s="1"/>
+      <x:c r="C62" s="1"/>
+      <x:c r="D62" s="1"/>
+      <x:c r="E62" s="1"/>
+      <x:c r="F62" s="1"/>
+      <x:c r="G62" s="1"/>
+      <x:c r="H62" s="1"/>
+      <x:c r="I62" s="1"/>
+      <x:c r="J62" s="1"/>
+      <x:c r="K62" s="1"/>
+      <x:c r="L62" s="1"/>
+    </x:row>
+    <x:row r="63" ht="22" customHeight="1">
+      <x:c r="A63" s="1"/>
+      <x:c r="B63" s="1"/>
+      <x:c r="C63" s="1"/>
+      <x:c r="D63" s="1"/>
+      <x:c r="E63" s="1"/>
+      <x:c r="F63" s="1"/>
+      <x:c r="G63" s="1"/>
+      <x:c r="H63" s="1"/>
+      <x:c r="I63" s="1"/>
+      <x:c r="J63" s="1"/>
+      <x:c r="K63" s="1"/>
+      <x:c r="L63" s="1"/>
+    </x:row>
+    <x:row r="64" ht="22" customHeight="1">
+      <x:c r="A64" s="1"/>
+      <x:c r="B64" s="1"/>
+      <x:c r="C64" s="1"/>
+      <x:c r="D64" s="1"/>
+      <x:c r="E64" s="1"/>
+      <x:c r="F64" s="1"/>
+      <x:c r="G64" s="1"/>
+      <x:c r="H64" s="1"/>
+      <x:c r="I64" s="1"/>
+      <x:c r="J64" s="1"/>
+      <x:c r="K64" s="1"/>
+      <x:c r="L64" s="1"/>
+    </x:row>
+    <x:row r="65" ht="22" customHeight="1">
+      <x:c r="A65" s="1"/>
+      <x:c r="B65" s="1"/>
+      <x:c r="C65" s="1"/>
+      <x:c r="D65" s="1"/>
+      <x:c r="E65" s="1"/>
+      <x:c r="F65" s="1"/>
+      <x:c r="G65" s="1"/>
+      <x:c r="H65" s="1"/>
+      <x:c r="I65" s="1"/>
+      <x:c r="J65" s="1"/>
+      <x:c r="K65" s="1"/>
+      <x:c r="L65" s="1"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="C4:I4"/>
+  </x:mergeCells>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="H7:H10">
+      <x:formula1>"Proposed,In progress,Completed,Blocked"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="3" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="3" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="42" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="17" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="17" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="17" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="17" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="17" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="17" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="17" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="17" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="17" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="22" customHeight="1">
+      <x:c r="A1" s="1"/>
+      <x:c r="B1" s="1"/>
+      <x:c r="C1" s="1"/>
+      <x:c r="D1" s="1"/>
+      <x:c r="E1" s="1"/>
+      <x:c r="F1" s="1"/>
+      <x:c r="G1" s="1"/>
+      <x:c r="H1" s="1"/>
+      <x:c r="I1" s="1"/>
+      <x:c r="J1" s="1"/>
+      <x:c r="K1" s="1"/>
+      <x:c r="L1" s="1"/>
+    </x:row>
+    <x:row r="2" ht="22" customHeight="1">
+      <x:c r="A2" s="1"/>
+      <x:c r="B2" s="1"/>
+      <x:c r="C2" s="2" t="str">
+        <x:v>Reconciliation checks</x:v>
+      </x:c>
+      <x:c r="D2" s="1"/>
+      <x:c r="E2" s="1"/>
+      <x:c r="F2" s="1"/>
+      <x:c r="G2" s="1"/>
+      <x:c r="H2" s="1"/>
+      <x:c r="I2" s="1"/>
+      <x:c r="J2" s="1"/>
+      <x:c r="K2" s="1"/>
+      <x:c r="L2" s="1"/>
+    </x:row>
+    <x:row r="3" ht="22" customHeight="1">
+      <x:c r="A3" s="1"/>
+      <x:c r="B3" s="1"/>
+      <x:c r="C3" s="3"/>
+      <x:c r="D3" s="3"/>
+      <x:c r="E3" s="3"/>
+      <x:c r="F3" s="3"/>
+      <x:c r="G3" s="3"/>
+      <x:c r="H3" s="3"/>
+      <x:c r="I3" s="3"/>
+      <x:c r="J3" s="3"/>
+      <x:c r="K3" s="3"/>
+      <x:c r="L3" s="3"/>
+    </x:row>
+    <x:row r="4" ht="22" customHeight="1">
+      <x:c r="A4" s="1"/>
+      <x:c r="B4" s="1"/>
+      <x:c r="C4" s="1"/>
+      <x:c r="D4" s="1"/>
+      <x:c r="E4" s="1"/>
+      <x:c r="F4" s="1"/>
+      <x:c r="G4" s="1"/>
+      <x:c r="H4" s="1"/>
+      <x:c r="I4" s="1"/>
+      <x:c r="J4" s="1"/>
+      <x:c r="K4" s="1"/>
+      <x:c r="L4" s="1"/>
+    </x:row>
+    <x:row r="5" ht="22" customHeight="1">
+      <x:c r="A5" s="1"/>
+      <x:c r="B5" s="1"/>
+      <x:c r="C5" s="1"/>
+      <x:c r="D5" s="1"/>
+      <x:c r="E5" s="1"/>
+      <x:c r="F5" s="1"/>
+      <x:c r="G5" s="1"/>
+      <x:c r="H5" s="1"/>
+      <x:c r="I5" s="1"/>
+      <x:c r="J5" s="1"/>
+      <x:c r="K5" s="1"/>
+      <x:c r="L5" s="1"/>
+    </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="1"/>
       <x:c r="B6" s="1"/>
@@ -6497,9 +9174,9 @@
       <x:c r="C7" s="5" t="str">
         <x:v>Replace incremental NPV</x:v>
       </x:c>
-      <x:c r="D7" s="38" t="n">
-        <x:f>'Summary'!F8-SUMPRODUCT('Cash Flows'!D31:I31,'Cash Flows'!D34:I34)</x:f>
-        <x:v>2.3283064365386963e-10</x:v>
+      <x:c r="D7" s="39" t="n">
+        <x:f>'Summary'!F8-SUMPRODUCT('After Tax'!D34:I34,'After Tax'!D28:I28)</x:f>
+        <x:v>2.0372681319713593e-10</x:v>
       </x:c>
       <x:c r="E7" s="39" t="n">
         <x:v>0.01</x:v>
@@ -6518,9 +9195,9 @@
       <x:c r="C8" s="5" t="str">
         <x:v>Lease incremental NPV</x:v>
       </x:c>
-      <x:c r="D8" s="38" t="n">
-        <x:f>'Summary'!F9-SUMPRODUCT('Cash Flows'!D32:I32,'Cash Flows'!D34:I34)</x:f>
-        <x:v>-2.3283064365386963e-10</x:v>
+      <x:c r="D8" s="39" t="n">
+        <x:f>'Summary'!F9-SUMPRODUCT('After Tax'!D35:I35,'After Tax'!D28:I28)</x:f>
+        <x:v>-1.7462298274040222e-10</x:v>
       </x:c>
       <x:c r="E8" s="39" t="n">
         <x:v>0.01</x:v>
@@ -6537,10 +9214,10 @@
       <x:c r="A9" s="1"/>
       <x:c r="B9" s="1"/>
       <x:c r="C9" s="5" t="str">
-        <x:v>Year 0 net cash</x:v>
-      </x:c>
-      <x:c r="D9" s="38" t="n">
-        <x:f>'Cash Flows'!D20+'Assumptions'!G9*('Assumptions'!G10-'Assumptions'!G11)</x:f>
+        <x:v>Loan repaid in year 5</x:v>
+      </x:c>
+      <x:c r="D9" s="39" t="n">
+        <x:f>'Financing'!I10</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E9" s="39" t="n">

</xml_diff>